<commit_message>
feat(checkout): automation Smart TV + refactor device-checkout page objects
- Them sheet Checkout_SmartTV (TC_SMARTTV.1-15) clone tu AP, chi doi label UI
- Promote AP page objects -> pages/common/device-* (class Device*Page) dung chung AP/Smart TV/Camera; xoa pages/ap rong
- AP spec: tham so hoa product qua env (AP_PRODUCT_*), repoint import sang common, fix locator TC_CKCOMMON.7 (.first())
- Them tests/smarttv/smarttv-checkout.spec.ts (TC_SMARTTV.*, default goi TV Samsung, env SMARTTV_PRODUCT_*)
- Fix duong dan report trong playwright.config.ts + package.json: ../../06_report -> ../06_report
- MEMORY checkout: ghi nhan Smart TV = clone rule AP (2026-06-08)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.1.xlsx
+++ b/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.1.xlsx
@@ -1,16 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Checkout_Common" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Checkout_Internet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Checkout_Camera" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Checkout_AP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Common" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Internet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_Camera" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_AP" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checkout_SmartTV" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -7619,4 +7620,846 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:L31"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="6" customWidth="1" style="31" min="1" max="1"/>
+    <col width="14" customWidth="1" style="31" min="2" max="2"/>
+    <col width="10" customWidth="1" style="31" min="3" max="3"/>
+    <col width="45" customWidth="1" style="31" min="4" max="5"/>
+    <col width="50" customWidth="1" style="31" min="6" max="6"/>
+    <col width="58" customWidth="1" style="31" min="7" max="7"/>
+    <col width="8" customWidth="1" style="31" min="8" max="8"/>
+    <col width="12" customWidth="1" style="31" min="9" max="9"/>
+    <col width="15" customWidth="1" style="31" min="10" max="10"/>
+    <col width="12" customWidth="1" style="31" min="11" max="11"/>
+    <col width="22.3" customWidth="1" style="31" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3" ht="15" customHeight="1" s="32">
+      <c r="C3" s="44" t="inlineStr">
+        <is>
+          <t>Mã chức năng:</t>
+        </is>
+      </c>
+      <c r="D3" s="44" t="inlineStr">
+        <is>
+          <t>TC_SMARTTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="32">
+      <c r="C4" s="44" t="inlineStr">
+        <is>
+          <t>Tên chức năng:</t>
+        </is>
+      </c>
+      <c r="D4" s="44" t="inlineStr">
+        <is>
+          <t>Đăng ký dịch vụ Smart TV — Checkout (số lượng + COD + địa chỉ lắp đặt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7" ht="30" customHeight="1" s="32">
+      <c r="A7" s="45" t="inlineStr">
+        <is>
+          <t>QC/AI</t>
+        </is>
+      </c>
+      <c r="B7" s="45" t="inlineStr">
+        <is>
+          <t>Testcase ID</t>
+        </is>
+      </c>
+      <c r="C7" s="45" t="inlineStr">
+        <is>
+          <t>Mức Độ Ưu Tiên</t>
+        </is>
+      </c>
+      <c r="D7" s="45" t="inlineStr">
+        <is>
+          <t>Nội Dung Test</t>
+        </is>
+      </c>
+      <c r="E7" s="45" t="inlineStr">
+        <is>
+          <t>Điều Kiện / Dữ Liệu Test</t>
+        </is>
+      </c>
+      <c r="F7" s="45" t="inlineStr">
+        <is>
+          <t>Các Bước Thực Hiện</t>
+        </is>
+      </c>
+      <c r="G7" s="45" t="inlineStr">
+        <is>
+          <t>Kết Quả Mong Đợi</t>
+        </is>
+      </c>
+      <c r="H7" s="45" t="inlineStr">
+        <is>
+          <t>Có thể
+Tự Động Hóa</t>
+        </is>
+      </c>
+      <c r="I7" s="45" t="inlineStr">
+        <is>
+          <t>Round 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19.5" customHeight="1" s="32">
+      <c r="I8" s="45" t="inlineStr">
+        <is>
+          <t>Kết Quả Thực Hiện</t>
+        </is>
+      </c>
+      <c r="J8" s="45" t="inlineStr">
+        <is>
+          <t>Người Thực Hiện</t>
+        </is>
+      </c>
+      <c r="K8" s="45" t="inlineStr">
+        <is>
+          <t>ID Bugs</t>
+        </is>
+      </c>
+      <c r="L8" s="45" t="inlineStr">
+        <is>
+          <t>Ghi Chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="32">
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>Lưu ý: Field validation (Họ tên, SĐT, Email, dropdown địa chỉ Tỉnh/Phường/Đường, popup Địa chỉ hành chính cũ, danh sách Phương thức thanh toán, luồng OTP) dùng chung — xem sheet Checkout_Common (TC_CKCOMMON). Sheet này chỉ kiểm tra phần ĐẶC THÙ dịch vụ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="32">
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>Lưu ý: Smart TV có rule GIỐNG HỆT AP (B1 chỉ chọn số lượng — không có chu kỳ; có địa chỉ lắp đặt; label giao hàng 3-7 ngày; KHÔNG có "Thời gian lắp đặt"), chỉ khác label hiển thị trên UI. Tham chiếu layout mockup Camera (camera.png). | v1.1 (2026-06-08): clone từ sheet Checkout_AP. Sản phẩm staging: Smart TV -TV SAMSUNG QA55Q60BAKXXV (4.500.000đ), slug tv-samsung-qa55q60bakxxv. Automation tái dùng spec AP (env AP_PRODUCT_SLUG/NAME/PRICE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="32">
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t>Nhóm 1: Hiển thị &amp; Điều hướng vào Checkout (số lượng — không chu kỳ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="55.2" customHeight="1" s="32">
+      <c r="A12" s="48" t="n"/>
+      <c r="B12" s="49">
+        <f>IF(D12="","",$D$3&amp;"."&amp;COUNTA($D$10:D12)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị tổng thể màn Checkout Smart TV (2 bước)</t>
+        </is>
+      </c>
+      <c r="E12" s="51" t="inlineStr">
+        <is>
+          <t>Đã chọn gói Smart TV ở màn Chi tiết</t>
+        </is>
+      </c>
+      <c r="F12" s="51" t="inlineStr">
+        <is>
+          <t>1. Quan sát tiến trình và bố cục màn checkout Smart TV</t>
+        </is>
+      </c>
+      <c r="G12" s="51" t="inlineStr">
+        <is>
+          <t>Header 2 bước: "Thanh toán" → "Hoàn tất đơn hàng"; hiển thị đủ block: Sản phẩm dịch vụ đã chọn, Thông tin cá nhân, Địa chỉ lắp đặt, Phương thức thanh toán, Thông tin khách hàng, Thông tin thanh toán</t>
+        </is>
+      </c>
+      <c r="H12" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="55.2" customHeight="1" s="32">
+      <c r="A13" s="48" t="n"/>
+      <c r="B13" s="49">
+        <f>IF(D13="","",$D$3&amp;"."&amp;COUNTA($D$10:D13)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C13" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn số lượng (không chu kỳ) rồi Mua ngay sang Checkout</t>
+        </is>
+      </c>
+      <c r="E13" s="51" t="inlineStr">
+        <is>
+          <t>Ở màn Chi tiết gói Smart TV</t>
+        </is>
+      </c>
+      <c r="F13" s="51" t="inlineStr">
+        <is>
+          <t>1. Chọn số lượng
+2. Click button "Mua ngay"</t>
+        </is>
+      </c>
+      <c r="G13" s="51" t="inlineStr">
+        <is>
+          <t>Điều hướng sang Thanh toán, load đúng tên gói + số lượng + số tiền</t>
+        </is>
+      </c>
+      <c r="H13" s="53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I13" s="56" t="n"/>
+      <c r="J13" s="56" t="n"/>
+      <c r="K13" s="56" t="n"/>
+      <c r="L13" s="55" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-Smart TV-00
+ (Smart TV không chu kỳ)
+→ đã cập nhất kết quả mong đợi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="55.2" customHeight="1" s="32">
+      <c r="A14" s="48" t="n"/>
+      <c r="B14" s="49">
+        <f>IF(D14="","",$D$3&amp;"."&amp;COUNTA($D$10:D14)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C14" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D14" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Sản phẩm dịch vụ đã chọn (không hiển thị chu kỳ)</t>
+        </is>
+      </c>
+      <c r="E14" s="51" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Smart TV</t>
+        </is>
+      </c>
+      <c r="F14" s="51" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block "Sản phẩm dịch vụ đã chọn"</t>
+        </is>
+      </c>
+      <c r="G14" s="51" t="inlineStr">
+        <is>
+          <t>Load đúng tên gói, số lượng, số tiền như màn hình chi tiết— KHÔNG hiển thị dòng chu kỳ</t>
+        </is>
+      </c>
+      <c r="H14" s="53" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I14" s="56" t="n"/>
+      <c r="J14" s="56" t="n"/>
+      <c r="K14" s="56" t="n"/>
+      <c r="L14" s="55" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-Smart TV-001 (Smart TV không chu kỳ)
+→ đã cập nhất kết quả mong đợi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="32">
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t>Nhóm 2: Block Địa chỉ lắp đặt (đặc thù Smart TV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="82.05" customHeight="1" s="32">
+      <c r="A16" s="57" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B16" s="58">
+        <f>IF(D16="","",$D$3&amp;"."&amp;COUNTA($D$10:D16)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="58" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Địa chỉ lắp đặt Smart TV hiển thị đúng các trường (không có Thời gian lắp đặt)</t>
+        </is>
+      </c>
+      <c r="E16" s="60" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Smart TV (B2)</t>
+        </is>
+      </c>
+      <c r="F16" s="60" t="inlineStr">
+        <is>
+          <t>1. Quan sát toàn bộ Block Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="G16" s="60" t="inlineStr">
+        <is>
+          <t>Block Địa chỉ lắp đặt hiển thị: link 'Địa chỉ trước sáp nhập', label cố định 'Thời gian giao hàng dự kiến từ 3 đến 7 ngày.', dropdown Tỉnh/Thành phố, dropdown Phường/Xã, dropdown Tên đường, textbox Số nhà, textbox Ghi chú. KHÔNG hiển thị trường 'Thời gian lắp đặt' (đặc thù Camera, Smart TV không có). Cơ chế validation dropdown/popup xem sheet Checkout_Common.</t>
+        </is>
+      </c>
+      <c r="H16" s="53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I16" s="56" t="n"/>
+      <c r="J16" s="56" t="n"/>
+      <c r="K16" s="56" t="inlineStr">
+        <is>
+          <t>Update – Unblock CLA-Smart TV-002 (Partially Resolved 2026-06-06): Smart TV có label giao hàng 3-7 ngày (cố định), KHÔNG có Thời gian lắp đặt. DOC-CK-05.</t>
+        </is>
+      </c>
+      <c r="L16" s="55" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-Smart TV-002 (note giao hàng/Thời gian lắp đặt Smart TV)
+→ tất cả dịch vụ đều khong có Thời gian lắp đặt</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1" s="32">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B17" s="61">
+        <f>IF(D17="","",$D$3&amp;"."&amp;COUNTA($D$10:D17)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D17" s="62" t="inlineStr">
+        <is>
+          <t>Kiểm tra label 'Thời gian giao hàng dự kiến từ 3 đến 7 ngày' hiển thị cố định trong Block Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="E17" s="62" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Smart TV (B2), Block Địa chỉ lắp đặt đang hiển thị</t>
+        </is>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <t>1. Quan sát nội dung Block Địa chỉ lắp đặt
+2. Thay đổi Tỉnh/Phường/Đường sang địa chỉ khác
+3. Quan sát lại label sau khi thay đổi địa chỉ</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr">
+        <is>
+          <t>Label 'Thời gian giao hàng dự kiến từ 3 đến 7 ngày.' hiển thị cố định trong Block Địa chỉ lắp đặt; text không thay đổi khi chọn địa chỉ khác hoặc theo bất kỳ điều kiện nào</t>
+        </is>
+      </c>
+      <c r="H17" s="31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K17" s="31" t="inlineStr">
+        <is>
+          <t>New – SC-Smart TV-019: Label giao hàng 3-7 ngày cố định xác nhận từ DOC-CK-05 (2026-06-06)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="32">
+      <c r="B18" s="63" t="inlineStr">
+        <is>
+          <t>Nhóm 3: Phương thức thanh toán &amp; Thông tin khách hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="41.75" customHeight="1" s="32">
+      <c r="A19" s="48" t="n"/>
+      <c r="B19" s="49">
+        <f>IF(D19="","",$D$3&amp;"."&amp;COUNTA($D$10:D19)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C19" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D19" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra Smart TV CÓ phương thức COD + online theo QLCS</t>
+        </is>
+      </c>
+      <c r="E19" s="51" t="inlineStr">
+        <is>
+          <t>Gói Smart TV cấu hình COD + online trên QLCS</t>
+        </is>
+      </c>
+      <c r="F19" s="51" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Phương thức thanh toán</t>
+        </is>
+      </c>
+      <c r="G19" s="51" t="inlineStr">
+        <is>
+          <t>Hiển thị COD "Thanh toán tại nhà" + các PTTT online theo QLCS; chỉ chọn 1; "Xem thêm" nếu &gt;4. Cơ chế danh sách PTTT xem TC_CKCOMMON</t>
+        </is>
+      </c>
+      <c r="H19" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="32">
+      <c r="A20" s="57" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B20" s="58">
+        <f>IF(D20="","",$D$3&amp;"."&amp;COUNTA($D$10:D20)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C20" s="58" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D20" s="59" t="inlineStr">
+        <is>
+          <t>Kiểm tra Block Thông tin khách hàng Smart TV auto-load (không có Thời gian lắp đặt)</t>
+        </is>
+      </c>
+      <c r="E20" s="60" t="inlineStr">
+        <is>
+          <t>Đã nhập đủ Thông tin cá nhân và Địa chỉ lắp đặt ở Block tương ứng</t>
+        </is>
+      </c>
+      <c r="F20" s="60" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Thông tin khách hàng</t>
+        </is>
+      </c>
+      <c r="G20" s="60" t="inlineStr">
+        <is>
+          <t>Block Thông tin khách hàng hiển thị: Họ tên, Số điện thoại, Địa chỉ tự động load theo dữ liệu đã nhập tại Block Thông tin cá nhân và Địa chỉ lắp đặt. KHÔNG hiển thị trường 'Thời gian lắp đặt' (Smart TV không có trường này, chỉ Camera mới có).</t>
+        </is>
+      </c>
+      <c r="H20" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I20" s="56" t="n"/>
+      <c r="J20" s="56" t="n"/>
+      <c r="K20" s="56" t="inlineStr">
+        <is>
+          <t>Update – Unblock CLA-Smart TV-002 (2026-06-06): Smart TV KHÔNG có Thời gian lắp đặt trong block TTKH. DOC-CK-05.</t>
+        </is>
+      </c>
+      <c r="L20" s="55" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-Smart TV-002 (Thời gian lắp đặt Smart TV)
+→ không cos thời gian lắp đwjt</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="32">
+      <c r="B21" s="63" t="inlineStr">
+        <is>
+          <t>Nhóm 4: Button Thanh toán &amp; Luồng thanh toán</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28.35" customHeight="1" s="32">
+      <c r="A22" s="48" t="n"/>
+      <c r="B22" s="49">
+        <f>IF(D22="","",$D$3&amp;"."&amp;COUNTA($D$10:D22)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C22" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D22" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi chính sách không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="E22" s="51" t="inlineStr">
+        <is>
+          <t>Gói/chính sách Smart TV không còn active trên QLCS</t>
+        </is>
+      </c>
+      <c r="F22" s="51" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G22" s="51" t="inlineStr">
+        <is>
+          <t>Báo lỗi chính sách không còn hiệu lực; KHÔNG thực hiện thanh toán</t>
+        </is>
+      </c>
+      <c r="H22" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="32">
+      <c r="A23" s="48" t="n"/>
+      <c r="B23" s="49">
+        <f>IF(D23="","",$D$3&amp;"."&amp;COUNTA($D$10:D23)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C23" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D23" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra Thanh toán khi data hợp lệ + chính sách active</t>
+        </is>
+      </c>
+      <c r="E23" s="51" t="inlineStr">
+        <is>
+          <t>Nhập đủ trường bắt buộc hợp lệ, chính sách active</t>
+        </is>
+      </c>
+      <c r="F23" s="51" t="inlineStr">
+        <is>
+          <t>1. Click button "Thanh toán"</t>
+        </is>
+      </c>
+      <c r="G23" s="51" t="inlineStr">
+        <is>
+          <t>Thực hiện luồng thanh toán theo PTTT đã chọn (COD → sang B3 luôn; Online → cổng 3rd party)</t>
+        </is>
+      </c>
+      <c r="H23" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="32">
+      <c r="B24" s="63" t="inlineStr">
+        <is>
+          <t>Nhóm 5: Bước Hoàn tất đơn hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="41.75" customHeight="1" s="32">
+      <c r="A25" s="48" t="n"/>
+      <c r="B25" s="49">
+        <f>IF(D25="","",$D$3&amp;"."&amp;COUNTA($D$10:D25)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C25" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D25" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT = COD</t>
+        </is>
+      </c>
+      <c r="E25" s="51" t="inlineStr">
+        <is>
+          <t>Chọn PTTT = COD, click Thanh toán</t>
+        </is>
+      </c>
+      <c r="F25" s="51" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất đặt hàng với PTTT = COD
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G25" s="51" t="inlineStr">
+        <is>
+          <t>Màn Hoàn tất: trạng thái "Chưa thanh toán" + nội dung "Đơn hàng đã đăng ký thành công. Kỹ thuật viên FPT sẽ liên hệ triển khai dịch vụ trong 8h-12h..."</t>
+        </is>
+      </c>
+      <c r="H25" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28.35" customHeight="1" s="32">
+      <c r="A26" s="48" t="n"/>
+      <c r="B26" s="49">
+        <f>IF(D26="","",$D$3&amp;"."&amp;COUNTA($D$10:D26)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C26" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D26" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra hoàn tất đơn hàng với PTTT Online thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="E26" s="51" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="F26" s="51" t="inlineStr">
+        <is>
+          <t>1. Hoàn tất thanh toán Online thành công
+2. Quan sát màn Hoàn tất</t>
+        </is>
+      </c>
+      <c r="G26" s="51" t="inlineStr">
+        <is>
+          <t>Bước "Hoàn tất đơn hàng" header màu xanh lá; trạng thái "Đã thanh toán" + nội dung thông báo thành công</t>
+        </is>
+      </c>
+      <c r="H26" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L26" s="31" t="inlineStr">
+        <is>
+          <t>case này tại sao auto không được ? Được chứ</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="32">
+      <c r="A27" s="48" t="n"/>
+      <c r="B27" s="49">
+        <f>IF(D27="","",$D$3&amp;"."&amp;COUNTA($D$10:D27)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C27" s="49" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D27" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra thanh toán Online thất bại quay về màn Thanh toán</t>
+        </is>
+      </c>
+      <c r="E27" s="51" t="inlineStr">
+        <is>
+          <t>Chọn PTTT Online, thanh toán thất bại</t>
+        </is>
+      </c>
+      <c r="F27" s="51" t="inlineStr">
+        <is>
+          <t>1. Thực hiện thanh toán Online thất bại</t>
+        </is>
+      </c>
+      <c r="G27" s="51" t="inlineStr">
+        <is>
+          <t>Quay về màn Thanh toán giữ nguyên thông tin đã chọn; CHỈ cho thay đổi PTTT + nhập mã ưu đãi, các trường còn lại disable</t>
+        </is>
+      </c>
+      <c r="H27" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L27" s="31" t="inlineStr">
+        <is>
+          <t>case này tại sao auto không được ? Được chứ</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="32">
+      <c r="B28" s="63" t="inlineStr">
+        <is>
+          <t>Nhóm 6: Mã ưu đãi &amp; Navigation &amp; Mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="41.75" customHeight="1" s="32">
+      <c r="A29" s="48" t="n"/>
+      <c r="B29" s="49">
+        <f>IF(D29="","",$D$3&amp;"."&amp;COUNTA($D$10:D29)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C29" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D29" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra áp dụng mã ưu đãi cho Smart TV</t>
+        </is>
+      </c>
+      <c r="E29" s="51" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Smart TV</t>
+        </is>
+      </c>
+      <c r="F29" s="51" t="inlineStr">
+        <is>
+          <t>1. Nhập/áp dụng mã ưu đãi</t>
+        </is>
+      </c>
+      <c r="G29" s="51" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm: voucher/mã ưu đãi chưa implement (như UltraFast)]. Kỳ vọng: trừ tiền</t>
+        </is>
+      </c>
+      <c r="H29" s="53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I29" s="56" t="n"/>
+      <c r="J29" s="56" t="n"/>
+      <c r="K29" s="56" t="n"/>
+      <c r="L29" s="55" t="inlineStr">
+        <is>
+          <t>BLOCKED – CLA-CAMAP-001 (voucher chưa implement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28.35" customHeight="1" s="32">
+      <c r="A30" s="48" t="n"/>
+      <c r="B30" s="49">
+        <f>IF(D30="","",$D$3&amp;"."&amp;COUNTA($D$10:D30)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C30" s="49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D30" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra button Quay lại điều hướng về màn Chi tiết gói</t>
+        </is>
+      </c>
+      <c r="E30" s="51" t="inlineStr">
+        <is>
+          <t>Đang ở màn Thanh toán Smart TV</t>
+        </is>
+      </c>
+      <c r="F30" s="51" t="inlineStr">
+        <is>
+          <t>1. Click button "Quay lại"</t>
+        </is>
+      </c>
+      <c r="G30" s="51" t="inlineStr">
+        <is>
+          <t>Điều hướng về màn Chi tiết gói Smart TV</t>
+        </is>
+      </c>
+      <c r="H30" s="49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28.35" customHeight="1" s="32">
+      <c r="A31" s="48" t="n"/>
+      <c r="B31" s="49">
+        <f>IF(D31="","",$D$3&amp;"."&amp;COUNTA($D$10:D31)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C31" s="49" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D31" s="50" t="inlineStr">
+        <is>
+          <t>Kiểm tra hiển thị luồng Checkout Smart TV trên mobile (≤ 768px)</t>
+        </is>
+      </c>
+      <c r="E31" s="51" t="inlineStr">
+        <is>
+          <t>Mở checkout Smart TV trên viewport mobile</t>
+        </is>
+      </c>
+      <c r="F31" s="51" t="inlineStr">
+        <is>
+          <t>1. Quan sát layout 2 bước + các block trên mobile</t>
+        </is>
+      </c>
+      <c r="G31" s="51" t="inlineStr">
+        <is>
+          <t>Các bước và block hiển thị đúng, không vỡ layout, thao tác được trên mobile</t>
+        </is>
+      </c>
+      <c r="H31" s="49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="17">
+    <mergeCell ref="B21:L21"/>
+    <mergeCell ref="B15:L15"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="B11:L11"/>
+    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="G7:G8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B28:L28"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="H7:H8"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="B18:L18"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: clean up gitkeep + normalize .gitignore line endings + update lock file
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.1.xlsx
+++ b/ecom-pdh/03_test-cases/functional/chucnang_checkout/AI_ISC_ecom-pdh_v1.1_TC_checkout_v1.1.xlsx
@@ -711,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A3:L105"/>
+  <dimension ref="A3:L98"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="31" min="1" max="1"/>
@@ -1042,51 +1042,21 @@
       <c r="L13" s="42" t="n"/>
     </row>
     <row r="14" ht="28.35" customHeight="1" s="32">
-      <c r="A14" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B14" s="40">
-        <f>IF(D14="","",$D$3&amp;"."&amp;COUNTA($D$10:D14)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C14" s="40" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="D14" s="43" t="inlineStr">
-        <is>
-          <t>Kiểm tra màu sắc mặc định tiến trình các bước và click vào bước khi đang ở Bước 1</t>
-        </is>
-      </c>
-      <c r="E14" s="43" t="inlineStr">
-        <is>
-          <t>- Đang ở Bước 1 màn hình nhập thông tin</t>
-        </is>
-      </c>
-      <c r="F14" s="43" t="inlineStr">
-        <is>
-          <t>1. Quan sát màu sắc các bước trên tiến trình
-2. Click lần lượt icon Bước 1, 2, 3</t>
-        </is>
-      </c>
-      <c r="G14" s="43" t="inlineStr">
-        <is>
-          <t>- Bước 1 màu xanh dương; Bước 2, 3 màu xám
-- Click các bước không có action, vẫn ở màn hình hiện tại</t>
-        </is>
-      </c>
-      <c r="H14" s="40" t="n"/>
-      <c r="I14" s="42" t="n"/>
-      <c r="J14" s="42" t="n"/>
-      <c r="K14" s="42" t="n"/>
-      <c r="L14" s="42" t="inlineStr">
-        <is>
-          <t>xóa case này giúp tôi</t>
-        </is>
-      </c>
+      <c r="B14" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 2: Block Thông tin cá nhân — Họ tên</t>
+        </is>
+      </c>
+      <c r="C14" s="35" t="n"/>
+      <c r="D14" s="35" t="n"/>
+      <c r="E14" s="35" t="n"/>
+      <c r="F14" s="35" t="n"/>
+      <c r="G14" s="35" t="n"/>
+      <c r="H14" s="35" t="n"/>
+      <c r="I14" s="35" t="n"/>
+      <c r="J14" s="35" t="n"/>
+      <c r="K14" s="35" t="n"/>
+      <c r="L14" s="36" t="n"/>
     </row>
     <row r="15" ht="28.35" customHeight="1" s="32">
       <c r="A15" s="39" t="inlineStr">
@@ -1100,55 +1070,88 @@
       </c>
       <c r="C15" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D15" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click Bước 1 khi đang ở Bước 2 (luồng nhiều bước)</t>
+          <t>Kiểm tra nhập Họ tên hợp lệ (có khoảng trắng đầu/cuối)</t>
         </is>
       </c>
       <c r="E15" s="41" t="inlineStr">
         <is>
-          <t>- Luồng checkout nhiều bước, đang ở Bước 2</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F15" s="41" t="inlineStr">
         <is>
-          <t>1. Click icon Bước 1 trên tiến trình</t>
+          <t>1. Nhập Họ tên hợp lệ chỉ gồm chữ + khoảng trắng, có khoảng trắng đầu/cuối
+2. Nhập các trường bắt buộc khác
+3. Submit</t>
         </is>
       </c>
       <c r="G15" s="41" t="inlineStr">
         <is>
-          <t>Cho phép quay về Bước 1</t>
-        </is>
-      </c>
-      <c r="H15" s="40" t="n"/>
+          <t>Chấp nhận, không báo lỗi; hệ thống tự trim khoảng trắng đầu/cuối khi submit</t>
+        </is>
+      </c>
+      <c r="H15" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I15" s="42" t="n"/>
       <c r="J15" s="42" t="n"/>
       <c r="K15" s="42" t="n"/>
-      <c r="L15" s="42" t="inlineStr">
-        <is>
-          <t>xóa case này giúp tôi</t>
-        </is>
-      </c>
+      <c r="L15" s="42" t="n"/>
     </row>
     <row r="16" ht="15" customHeight="1" s="32">
-      <c r="B16" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 2: Block Sản phẩm dịch vụ đã chọn</t>
-        </is>
-      </c>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="35" t="n"/>
-      <c r="F16" s="35" t="n"/>
-      <c r="G16" s="35" t="n"/>
-      <c r="H16" s="35" t="n"/>
-      <c r="I16" s="35" t="n"/>
-      <c r="J16" s="35" t="n"/>
-      <c r="K16" s="35" t="n"/>
-      <c r="L16" s="36" t="n"/>
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B16" s="40">
+        <f>IF(D16="","",$D$3&amp;"."&amp;COUNTA($D$10:D16)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C16" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra Họ tên để trống hoặc chỉ khoảng trắng</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>1. Để trống (hoặc nhập khoảng trắng) trường Họ tên
+2. Click ra ngoài trường</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>Border đỏ trường Họ tên và hiển thị "Vui lòng nhập họ tên."</t>
+        </is>
+      </c>
+      <c r="H16" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I16" s="42" t="n"/>
+      <c r="J16" s="42" t="n"/>
+      <c r="K16" s="42" t="n"/>
+      <c r="L16" s="42" t="n"/>
     </row>
     <row r="17" ht="28.35" customHeight="1" s="32">
       <c r="A17" s="39" t="inlineStr">
@@ -1162,27 +1165,29 @@
       </c>
       <c r="C17" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D17" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Block Sản phẩm dịch vụ đã chọn load đúng thông tin</t>
+          <t>Kiểm tra Họ tên chứa số hoặc ký tự đặc biệt</t>
         </is>
       </c>
       <c r="E17" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn gói dịch vụ cụ thể (tên, chu kỳ, số lượng, giá) ở màn Chi tiết</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F17" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát Block Sản phẩm dịch vụ đã chọn</t>
+          <t>1. Nhập/paste Họ tên có chứa số hoặc ký tự đặc biệt
+2. Click ra ngoài trường</t>
         </is>
       </c>
       <c r="G17" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị đúng: số lượng, tên gói, chu kỳ (VD 3/6/12 tháng), giá (sau ưu đãi nếu có), icon theo config Product Hub</t>
+          <t>Hiển thị "Họ tên không hợp lệ." (chỉ cho phép chữ + khoảng trắng)</t>
         </is>
       </c>
       <c r="H17" s="40" t="inlineStr">
@@ -1193,28 +1198,53 @@
       <c r="I17" s="42" t="n"/>
       <c r="J17" s="42" t="n"/>
       <c r="K17" s="42" t="n"/>
-      <c r="L17" s="42" t="inlineStr">
-        <is>
-          <t>bỏ nhóm 2 và case này, case này check riêng từng dịch vụ</t>
-        </is>
-      </c>
+      <c r="L17" s="42" t="n"/>
     </row>
     <row r="18" ht="15" customHeight="1" s="32">
-      <c r="B18" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 3: Block Thông tin cá nhân — Họ tên</t>
-        </is>
-      </c>
-      <c r="C18" s="35" t="n"/>
-      <c r="D18" s="35" t="n"/>
-      <c r="E18" s="35" t="n"/>
-      <c r="F18" s="35" t="n"/>
-      <c r="G18" s="35" t="n"/>
-      <c r="H18" s="35" t="n"/>
-      <c r="I18" s="35" t="n"/>
-      <c r="J18" s="35" t="n"/>
-      <c r="K18" s="35" t="n"/>
-      <c r="L18" s="36" t="n"/>
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B18" s="40">
+        <f>IF(D18="","",$D$3&amp;"."&amp;COUNTA($D$10:D18)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D18" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra Họ tên nhập/paste vượt quá 100 ký tự</t>
+        </is>
+      </c>
+      <c r="E18" s="41" t="inlineStr">
+        <is>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
+        </is>
+      </c>
+      <c r="F18" s="41" t="inlineStr">
+        <is>
+          <t>1. Nhập/paste Họ tên dài hơn 100 ký tự</t>
+        </is>
+      </c>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>Chỉ cho nhập và hiển thị tối đa 100 ký tự</t>
+        </is>
+      </c>
+      <c r="H18" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I18" s="42" t="n"/>
+      <c r="J18" s="42" t="n"/>
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="42" t="n"/>
     </row>
     <row r="19" ht="55.2" customHeight="1" s="32">
       <c r="A19" s="39" t="inlineStr">
@@ -1228,12 +1258,12 @@
       </c>
       <c r="C19" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D19" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra nhập Họ tên hợp lệ (có khoảng trắng đầu/cuối)</t>
+          <t>Kiểm tra icon X hiển thị và xóa dữ liệu trường Họ tên</t>
         </is>
       </c>
       <c r="E19" s="41" t="inlineStr">
@@ -1244,14 +1274,13 @@
       </c>
       <c r="F19" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập Họ tên hợp lệ chỉ gồm chữ + khoảng trắng, có khoảng trắng đầu/cuối
-2. Nhập các trường bắt buộc khác
-3. Submit</t>
+          <t>1. Nhập ký tự bất kỳ vào Họ tên
+2. Click icon X cuối textbox</t>
         </is>
       </c>
       <c r="G19" s="41" t="inlineStr">
         <is>
-          <t>Chấp nhận, không báo lỗi; hệ thống tự trim khoảng trắng đầu/cuối khi submit</t>
+          <t>Icon X hiển thị khi có dữ liệu; click X xóa toàn bộ và ẩn icon X</t>
         </is>
       </c>
       <c r="H19" s="40" t="inlineStr">
@@ -1265,87 +1294,56 @@
       <c r="L19" s="42" t="n"/>
     </row>
     <row r="20" ht="41.75" customHeight="1" s="32">
-      <c r="A20" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B20" s="40">
-        <f>IF(D20="","",$D$3&amp;"."&amp;COUNTA($D$10:D20)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C20" s="40" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 3: Block Thông tin cá nhân — Số điện thoại</t>
+        </is>
+      </c>
+      <c r="C20" s="35" t="n"/>
+      <c r="D20" s="35" t="n"/>
+      <c r="E20" s="35" t="n"/>
+      <c r="F20" s="35" t="n"/>
+      <c r="G20" s="35" t="n"/>
+      <c r="H20" s="35" t="n"/>
+      <c r="I20" s="35" t="n"/>
+      <c r="J20" s="35" t="n"/>
+      <c r="K20" s="35" t="n"/>
+      <c r="L20" s="36" t="n"/>
+    </row>
+    <row r="21" ht="41.75" customHeight="1" s="32">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B21" s="40">
+        <f>IF(D21="","",$D$3&amp;"."&amp;COUNTA($D$10:D21)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D20" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra Họ tên để trống hoặc chỉ khoảng trắng</t>
-        </is>
-      </c>
-      <c r="E20" s="41" t="inlineStr">
+      <c r="D21" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra nhập Số điện thoại hợp lệ</t>
+        </is>
+      </c>
+      <c r="E21" s="41" t="inlineStr">
         <is>
           <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
 - Đang ở màn hình Checkout</t>
         </is>
       </c>
-      <c r="F20" s="41" t="inlineStr">
-        <is>
-          <t>1. Để trống (hoặc nhập khoảng trắng) trường Họ tên
-2. Click ra ngoài trường</t>
-        </is>
-      </c>
-      <c r="G20" s="41" t="inlineStr">
-        <is>
-          <t>Border đỏ trường Họ tên và hiển thị "Vui lòng nhập họ tên."</t>
-        </is>
-      </c>
-      <c r="H20" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I20" s="42" t="n"/>
-      <c r="J20" s="42" t="n"/>
-      <c r="K20" s="42" t="n"/>
-      <c r="L20" s="42" t="n"/>
-    </row>
-    <row r="21" ht="41.75" customHeight="1" s="32">
-      <c r="A21" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B21" s="40">
-        <f>IF(D21="","",$D$3&amp;"."&amp;COUNTA($D$10:D21)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C21" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D21" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra Họ tên chứa số hoặc ký tự đặc biệt</t>
-        </is>
-      </c>
-      <c r="E21" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
-        </is>
-      </c>
       <c r="F21" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập/paste Họ tên có chứa số hoặc ký tự đặc biệt
-2. Click ra ngoài trường</t>
+          <t>1. Nhập SĐT 10 số bắt đầu bằng 0 (VD 0901234567)</t>
         </is>
       </c>
       <c r="G21" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị "Họ tên không hợp lệ." (chỉ cho phép chữ + khoảng trắng)</t>
+          <t>Chấp nhận, không báo lỗi; icon X hiển thị cuối textbox</t>
         </is>
       </c>
       <c r="H21" s="40" t="inlineStr">
@@ -1370,12 +1368,12 @@
       </c>
       <c r="C22" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D22" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Họ tên nhập/paste vượt quá 100 ký tự</t>
+          <t>Kiểm tra Số điện thoại để trống</t>
         </is>
       </c>
       <c r="E22" s="41" t="inlineStr">
@@ -1386,12 +1384,13 @@
       </c>
       <c r="F22" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập/paste Họ tên dài hơn 100 ký tự</t>
+          <t>1. Để trống trường Số điện thoại
+2. Click ra ngoài (hoặc submit)</t>
         </is>
       </c>
       <c r="G22" s="41" t="inlineStr">
         <is>
-          <t>Chỉ cho nhập và hiển thị tối đa 100 ký tự</t>
+          <t>Border đỏ và hiển thị "Vui lòng nhập số điện thoại."</t>
         </is>
       </c>
       <c r="H22" s="40" t="inlineStr">
@@ -1416,12 +1415,12 @@
       </c>
       <c r="C23" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D23" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra icon X hiển thị và xóa dữ liệu trường Họ tên</t>
+          <t>Kiểm tra Số điện thoại chứa ký tự không phải số</t>
         </is>
       </c>
       <c r="E23" s="41" t="inlineStr">
@@ -1432,13 +1431,12 @@
       </c>
       <c r="F23" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập ký tự bất kỳ vào Họ tên
-2. Click icon X cuối textbox</t>
+          <t>1. Nhập/paste SĐT có ký tự không phải số</t>
         </is>
       </c>
       <c r="G23" s="41" t="inlineStr">
         <is>
-          <t>Icon X hiển thị khi có dữ liệu; click X xóa toàn bộ và ẩn icon X</t>
+          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
         </is>
       </c>
       <c r="H23" s="40" t="inlineStr">
@@ -1452,21 +1450,50 @@
       <c r="L23" s="42" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="32">
-      <c r="B24" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 4: Block Thông tin cá nhân — Số điện thoại</t>
-        </is>
-      </c>
-      <c r="C24" s="35" t="n"/>
-      <c r="D24" s="35" t="n"/>
-      <c r="E24" s="35" t="n"/>
-      <c r="F24" s="35" t="n"/>
-      <c r="G24" s="35" t="n"/>
-      <c r="H24" s="35" t="n"/>
-      <c r="I24" s="35" t="n"/>
-      <c r="J24" s="35" t="n"/>
-      <c r="K24" s="35" t="n"/>
-      <c r="L24" s="36" t="n"/>
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B24" s="40">
+        <f>IF(D24="","",$D$3&amp;"."&amp;COUNTA($D$10:D24)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C24" s="40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D24" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra Số điện thoại 10 số nhưng không bắt đầu bằng 0</t>
+        </is>
+      </c>
+      <c r="E24" s="41" t="inlineStr">
+        <is>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
+        </is>
+      </c>
+      <c r="F24" s="41" t="inlineStr">
+        <is>
+          <t>1. Nhập SĐT 10 số bắt đầu khác 0 (VD 1901234567)</t>
+        </is>
+      </c>
+      <c r="G24" s="41" t="inlineStr">
+        <is>
+          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
+        </is>
+      </c>
+      <c r="H24" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I24" s="42" t="n"/>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
     </row>
     <row r="25" ht="41.75" customHeight="1" s="32">
       <c r="A25" s="39" t="inlineStr">
@@ -1480,12 +1507,12 @@
       </c>
       <c r="C25" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D25" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra nhập Số điện thoại hợp lệ</t>
+          <t>Kiểm tra Số điện thoại nhập/paste nhiều hơn 10 số</t>
         </is>
       </c>
       <c r="E25" s="41" t="inlineStr">
@@ -1496,12 +1523,12 @@
       </c>
       <c r="F25" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập SĐT 10 số bắt đầu bằng 0 (VD 0901234567)</t>
+          <t>1. Nhập/paste SĐT nhiều hơn 10 chữ số</t>
         </is>
       </c>
       <c r="G25" s="41" t="inlineStr">
         <is>
-          <t>Chấp nhận, không báo lỗi; icon X hiển thị cuối textbox</t>
+          <t>Chỉ nhận 10 số đầu, tự cắt bỏ từ số thứ 11</t>
         </is>
       </c>
       <c r="H25" s="40" t="inlineStr">
@@ -1526,12 +1553,12 @@
       </c>
       <c r="C26" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D26" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Số điện thoại để trống</t>
+          <t>Kiểm tra icon X xóa dữ liệu trường Số điện thoại</t>
         </is>
       </c>
       <c r="E26" s="41" t="inlineStr">
@@ -1542,13 +1569,13 @@
       </c>
       <c r="F26" s="41" t="inlineStr">
         <is>
-          <t>1. Để trống trường Số điện thoại
-2. Click ra ngoài (hoặc submit)</t>
+          <t>1. Nhập ký tự vào SĐT
+2. Click icon X</t>
         </is>
       </c>
       <c r="G26" s="41" t="inlineStr">
         <is>
-          <t>Border đỏ và hiển thị "Vui lòng nhập số điện thoại."</t>
+          <t>Xóa toàn bộ dữ liệu SĐT và ẩn icon X</t>
         </is>
       </c>
       <c r="H26" s="40" t="inlineStr">
@@ -1562,50 +1589,21 @@
       <c r="L26" s="42" t="n"/>
     </row>
     <row r="27" ht="41.75" customHeight="1" s="32">
-      <c r="A27" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B27" s="40">
-        <f>IF(D27="","",$D$3&amp;"."&amp;COUNTA($D$10:D27)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C27" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D27" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra Số điện thoại chứa ký tự không phải số</t>
-        </is>
-      </c>
-      <c r="E27" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
-        </is>
-      </c>
-      <c r="F27" s="41" t="inlineStr">
-        <is>
-          <t>1. Nhập/paste SĐT có ký tự không phải số</t>
-        </is>
-      </c>
-      <c r="G27" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
-        </is>
-      </c>
-      <c r="H27" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I27" s="42" t="n"/>
-      <c r="J27" s="42" t="n"/>
-      <c r="K27" s="42" t="n"/>
-      <c r="L27" s="42" t="n"/>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 4: Block Thông tin cá nhân — Email (chỉ Hyperfast/UltraFast)</t>
+        </is>
+      </c>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="35" t="n"/>
+      <c r="G27" s="35" t="n"/>
+      <c r="H27" s="35" t="n"/>
+      <c r="I27" s="35" t="n"/>
+      <c r="J27" s="35" t="n"/>
+      <c r="K27" s="35" t="n"/>
+      <c r="L27" s="36" t="n"/>
     </row>
     <row r="28" ht="41.75" customHeight="1" s="32">
       <c r="A28" s="39" t="inlineStr">
@@ -1624,23 +1622,23 @@
       </c>
       <c r="D28" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Số điện thoại 10 số nhưng không bắt đầu bằng 0</t>
+          <t>Kiểm tra trường Email placeholder và cho phép để trống</t>
         </is>
       </c>
       <c r="E28" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
         </is>
       </c>
       <c r="F28" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập SĐT 10 số bắt đầu khác 0 (VD 1901234567)</t>
+          <t>1. Quan sát placeholder trường Email
+2. Để trống Email rồi click ra ngoài</t>
         </is>
       </c>
       <c r="G28" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị "Số điện thoại không hợp lệ."</t>
+          <t>Placeholder "Nhập email"; cho phép để trống, không báo lỗi (Email không bắt buộc)</t>
         </is>
       </c>
       <c r="H28" s="40" t="inlineStr">
@@ -1670,23 +1668,23 @@
       </c>
       <c r="D29" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Số điện thoại nhập/paste nhiều hơn 10 số</t>
+          <t>Kiểm tra nhập Email sai định dạng</t>
         </is>
       </c>
       <c r="E29" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
         </is>
       </c>
       <c r="F29" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập/paste SĐT nhiều hơn 10 chữ số</t>
+          <t>1. Nhập Email sai định dạng (VD: email_sai_format)
+2. Click ra ngoài</t>
         </is>
       </c>
       <c r="G29" s="41" t="inlineStr">
         <is>
-          <t>Chỉ nhận 10 số đầu, tự cắt bỏ từ số thứ 11</t>
+          <t>Hiển thị "Email không hợp lệ"</t>
         </is>
       </c>
       <c r="H29" s="40" t="inlineStr">
@@ -1711,29 +1709,28 @@
       </c>
       <c r="C30" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D30" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra icon X xóa dữ liệu trường Số điện thoại</t>
+          <t>Kiểm tra nhập Email không có domain</t>
         </is>
       </c>
       <c r="E30" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
         </is>
       </c>
       <c r="F30" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập ký tự vào SĐT
-2. Click icon X</t>
+          <t>1. Nhập Email không có domain (VD: test@)
+2. Click ra ngoài</t>
         </is>
       </c>
       <c r="G30" s="41" t="inlineStr">
         <is>
-          <t>Xóa toàn bộ dữ liệu SĐT và ẩn icon X</t>
+          <t>Hiển thị "Email không hợp lệ"</t>
         </is>
       </c>
       <c r="H30" s="40" t="inlineStr">
@@ -1747,67 +1744,68 @@
       <c r="L30" s="42" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="32">
-      <c r="B31" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 5: Block Thông tin cá nhân — Email (chỉ Hyperfast/UltraFast)</t>
-        </is>
-      </c>
-      <c r="C31" s="35" t="n"/>
-      <c r="D31" s="35" t="n"/>
-      <c r="E31" s="35" t="n"/>
-      <c r="F31" s="35" t="n"/>
-      <c r="G31" s="35" t="n"/>
-      <c r="H31" s="35" t="n"/>
-      <c r="I31" s="35" t="n"/>
-      <c r="J31" s="35" t="n"/>
-      <c r="K31" s="35" t="n"/>
-      <c r="L31" s="36" t="n"/>
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B31" s="40">
+        <f>IF(D31="","",$D$3&amp;"."&amp;COUNTA($D$10:D31)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D31" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra Email hiển thị realtime sang block Thông tin khách hàng và icon X</t>
+        </is>
+      </c>
+      <c r="E31" s="41" t="inlineStr">
+        <is>
+          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
+        </is>
+      </c>
+      <c r="F31" s="41" t="inlineStr">
+        <is>
+          <t>1. Nhập Email hợp lệ (VD: Acb@gmail.com)
+2. Quan sát block Thông tin khách hàng
+3. Click icon X</t>
+        </is>
+      </c>
+      <c r="G31" s="41" t="inlineStr">
+        <is>
+          <t>Email hiển thị realtime sang block Thông tin khách hàng; icon X xóa được Email</t>
+        </is>
+      </c>
+      <c r="H31" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I31" s="42" t="n"/>
+      <c r="J31" s="42" t="n"/>
+      <c r="K31" s="42" t="n"/>
+      <c r="L31" s="42" t="n"/>
     </row>
     <row r="32" ht="28.35" customHeight="1" s="32">
-      <c r="A32" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B32" s="40">
-        <f>IF(D32="","",$D$3&amp;"."&amp;COUNTA($D$10:D32)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C32" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D32" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra trường Email placeholder và cho phép để trống</t>
-        </is>
-      </c>
-      <c r="E32" s="41" t="inlineStr">
-        <is>
-          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
-        </is>
-      </c>
-      <c r="F32" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát placeholder trường Email
-2. Để trống Email rồi click ra ngoài</t>
-        </is>
-      </c>
-      <c r="G32" s="41" t="inlineStr">
-        <is>
-          <t>Placeholder "Nhập email"; cho phép để trống, không báo lỗi (Email không bắt buộc)</t>
-        </is>
-      </c>
-      <c r="H32" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I32" s="42" t="n"/>
-      <c r="J32" s="42" t="n"/>
-      <c r="K32" s="42" t="n"/>
-      <c r="L32" s="42" t="n"/>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 5: Block Địa chỉ lắp đặt — Tỉnh/Thành phố &amp; pre-fill</t>
+        </is>
+      </c>
+      <c r="C32" s="35" t="n"/>
+      <c r="D32" s="35" t="n"/>
+      <c r="E32" s="35" t="n"/>
+      <c r="F32" s="35" t="n"/>
+      <c r="G32" s="35" t="n"/>
+      <c r="H32" s="35" t="n"/>
+      <c r="I32" s="35" t="n"/>
+      <c r="J32" s="35" t="n"/>
+      <c r="K32" s="35" t="n"/>
+      <c r="L32" s="36" t="n"/>
     </row>
     <row r="33" ht="28.35" customHeight="1" s="32">
       <c r="A33" s="39" t="inlineStr">
@@ -1821,28 +1819,28 @@
       </c>
       <c r="C33" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D33" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra nhập Email sai định dạng</t>
+          <t>Kiểm tra Tỉnh/Thành phố mặc định rỗng và placeholder</t>
         </is>
       </c>
       <c r="E33" s="41" t="inlineStr">
         <is>
-          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F33" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập Email sai định dạng (VD: email_sai_format)
-2. Click ra ngoài</t>
+          <t>1. Quan sát trường Tỉnh/Thành phố khi chưa chọn</t>
         </is>
       </c>
       <c r="G33" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị "Email không hợp lệ"</t>
+          <t>Mặc định rỗng; placeholder "Chọn tỉnh/thành phố"</t>
         </is>
       </c>
       <c r="H33" s="40" t="inlineStr">
@@ -1872,23 +1870,24 @@
       </c>
       <c r="D34" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra nhập Email không có domain</t>
+          <t>Kiểm tra không chọn Tỉnh/Thành phố</t>
         </is>
       </c>
       <c r="E34" s="41" t="inlineStr">
         <is>
-          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F34" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập Email không có domain (VD: test@)
-2. Click ra ngoài</t>
+          <t>1. Click trường Tỉnh/Thành phố
+2. Không chọn và click ra ngoài</t>
         </is>
       </c>
       <c r="G34" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị "Email không hợp lệ"</t>
+          <t>Border đỏ và hiển thị "Vui lòng chọn tỉnh/thành phố."</t>
         </is>
       </c>
       <c r="H34" s="40" t="inlineStr">
@@ -1918,24 +1917,23 @@
       </c>
       <c r="D35" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Email hiển thị realtime sang block Thông tin khách hàng và icon X</t>
+          <t>Kiểm tra load danh sách Tỉnh/Thành phố theo ĐCHC mới</t>
         </is>
       </c>
       <c r="E35" s="41" t="inlineStr">
         <is>
-          <t>- Đang Checkout dịch vụ Hyperfast/UltraFast</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F35" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập Email hợp lệ (VD: Acb@gmail.com)
-2. Quan sát block Thông tin khách hàng
-3. Click icon X</t>
+          <t>1. Click dropdown Tỉnh/Thành phố</t>
         </is>
       </c>
       <c r="G35" s="41" t="inlineStr">
         <is>
-          <t>Email hiển thị realtime sang block Thông tin khách hàng; icon X xóa được Email</t>
+          <t>Hiển thị đủ tỉnh/thành toàn quốc theo ĐCHC mới; HCM, HN, Đà Nẵng load đầu danh sách</t>
         </is>
       </c>
       <c r="H35" s="40" t="inlineStr">
@@ -1949,21 +1947,51 @@
       <c r="L35" s="42" t="n"/>
     </row>
     <row r="36" ht="15" customHeight="1" s="32">
-      <c r="B36" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 6: Block Địa chỉ lắp đặt — Tỉnh/Thành phố &amp; pre-fill</t>
-        </is>
-      </c>
-      <c r="C36" s="35" t="n"/>
-      <c r="D36" s="35" t="n"/>
-      <c r="E36" s="35" t="n"/>
-      <c r="F36" s="35" t="n"/>
-      <c r="G36" s="35" t="n"/>
-      <c r="H36" s="35" t="n"/>
-      <c r="I36" s="35" t="n"/>
-      <c r="J36" s="35" t="n"/>
-      <c r="K36" s="35" t="n"/>
-      <c r="L36" s="36" t="n"/>
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B36" s="40">
+        <f>IF(D36="","",$D$3&amp;"."&amp;COUNTA($D$10:D36)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C36" s="40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D36" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra tìm kiếm Tỉnh/Thành phố</t>
+        </is>
+      </c>
+      <c r="E36" s="41" t="inlineStr">
+        <is>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
+        </is>
+      </c>
+      <c r="F36" s="41" t="inlineStr">
+        <is>
+          <t>1. Click dropdown Tỉnh/Thành phố
+2. Nhập từ khóa cần tìm</t>
+        </is>
+      </c>
+      <c r="G36" s="41" t="inlineStr">
+        <is>
+          <t>Hiển thị danh sách khớp từ khóa (quy tắc contains)</t>
+        </is>
+      </c>
+      <c r="H36" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I36" s="42" t="n"/>
+      <c r="J36" s="42" t="n"/>
+      <c r="K36" s="42" t="n"/>
+      <c r="L36" s="42" t="n"/>
     </row>
     <row r="37" ht="41.75" customHeight="1" s="32">
       <c r="A37" s="39" t="inlineStr">
@@ -1977,12 +2005,12 @@
       </c>
       <c r="C37" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D37" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Tỉnh/Thành phố mặc định rỗng và placeholder</t>
+          <t>Kiểm tra chọn Tỉnh/Thành phố load thêm trường địa chỉ</t>
         </is>
       </c>
       <c r="E37" s="41" t="inlineStr">
@@ -1993,12 +2021,12 @@
       </c>
       <c r="F37" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát trường Tỉnh/Thành phố khi chưa chọn</t>
+          <t>1. Chọn 1 Tỉnh/Thành phố bất kỳ</t>
         </is>
       </c>
       <c r="G37" s="41" t="inlineStr">
         <is>
-          <t>Mặc định rỗng; placeholder "Chọn tỉnh/thành phố"</t>
+          <t>Chỉ chọn được 1; load thêm Phường/Xã, Tên đường, Số nhà, Ghi chú</t>
         </is>
       </c>
       <c r="H37" s="40" t="inlineStr">
@@ -2028,24 +2056,22 @@
       </c>
       <c r="D38" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra không chọn Tỉnh/Thành phố</t>
+          <t>Kiểm tra đổi Tỉnh/Thành phố reload các trường phụ thuộc</t>
         </is>
       </c>
       <c r="E38" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đã chọn 1 Tỉnh/Thành phố</t>
         </is>
       </c>
       <c r="F38" s="41" t="inlineStr">
         <is>
-          <t>1. Click trường Tỉnh/Thành phố
-2. Không chọn và click ra ngoài</t>
+          <t>1. Chọn 1 Tỉnh/Thành phố khác</t>
         </is>
       </c>
       <c r="G38" s="41" t="inlineStr">
         <is>
-          <t>Border đỏ và hiển thị "Vui lòng chọn tỉnh/thành phố."</t>
+          <t>Reload Phường/Xã tương ứng, reset Tên đường, trigger kiểm tra chính sách giá</t>
         </is>
       </c>
       <c r="H38" s="40" t="inlineStr">
@@ -2075,23 +2101,23 @@
       </c>
       <c r="D39" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra load danh sách Tỉnh/Thành phố theo ĐCHC mới</t>
+          <t>Kiểm tra pre-fill "Địa chỉ trước sáp nhập" điền toàn bộ địa chỉ</t>
         </is>
       </c>
       <c r="E39" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Account đã có địa chỉ lưu sẵn từ đơn trước
+- Dịch vụ có link "Địa chỉ trước sáp nhập"</t>
         </is>
       </c>
       <c r="F39" s="41" t="inlineStr">
         <is>
-          <t>1. Click dropdown Tỉnh/Thành phố</t>
+          <t>1. Click link "Địa chỉ trước sáp nhập"</t>
         </is>
       </c>
       <c r="G39" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị đủ tỉnh/thành toàn quốc theo ĐCHC mới; HCM, HN, Đà Nẵng load đầu danh sách</t>
+          <t>Hệ thống tự điền TOÀN BỘ địa chỉ đã lưu (Tỉnh/TP, Phường/Xã, Tên đường, Số nhà...)</t>
         </is>
       </c>
       <c r="H39" s="40" t="inlineStr">
@@ -2105,51 +2131,21 @@
       <c r="L39" s="42" t="n"/>
     </row>
     <row r="40" ht="41.75" customHeight="1" s="32">
-      <c r="A40" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B40" s="40">
-        <f>IF(D40="","",$D$3&amp;"."&amp;COUNTA($D$10:D40)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D40" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra tìm kiếm Tỉnh/Thành phố</t>
-        </is>
-      </c>
-      <c r="E40" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
-        </is>
-      </c>
-      <c r="F40" s="41" t="inlineStr">
-        <is>
-          <t>1. Click dropdown Tỉnh/Thành phố
-2. Nhập từ khóa cần tìm</t>
-        </is>
-      </c>
-      <c r="G40" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị danh sách khớp từ khóa (quy tắc contains)</t>
-        </is>
-      </c>
-      <c r="H40" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I40" s="42" t="n"/>
-      <c r="J40" s="42" t="n"/>
-      <c r="K40" s="42" t="n"/>
-      <c r="L40" s="42" t="n"/>
+      <c r="B40" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 6: Block Địa chỉ lắp đặt — Phường/Xã &amp; kiểm tra chính sách giá</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="n"/>
+      <c r="D40" s="35" t="n"/>
+      <c r="E40" s="35" t="n"/>
+      <c r="F40" s="35" t="n"/>
+      <c r="G40" s="35" t="n"/>
+      <c r="H40" s="35" t="n"/>
+      <c r="I40" s="35" t="n"/>
+      <c r="J40" s="35" t="n"/>
+      <c r="K40" s="35" t="n"/>
+      <c r="L40" s="36" t="n"/>
     </row>
     <row r="41" ht="41.75" customHeight="1" s="32">
       <c r="A41" s="39" t="inlineStr">
@@ -2168,23 +2164,23 @@
       </c>
       <c r="D41" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra chọn Tỉnh/Thành phố load thêm trường địa chỉ</t>
+          <t>Kiểm tra Phường/Xã placeholder và bắt buộc chọn</t>
         </is>
       </c>
       <c r="E41" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đã chọn Tỉnh/Thành phố</t>
         </is>
       </c>
       <c r="F41" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn 1 Tỉnh/Thành phố bất kỳ</t>
+          <t>1. Quan sát placeholder Phường/Xã
+2. Không chọn và click ra ngoài</t>
         </is>
       </c>
       <c r="G41" s="41" t="inlineStr">
         <is>
-          <t>Chỉ chọn được 1; load thêm Phường/Xã, Tên đường, Số nhà, Ghi chú</t>
+          <t>Placeholder "Chọn phường/xã"; border đỏ + "Vui lòng chọn phường/xã."</t>
         </is>
       </c>
       <c r="H41" s="40" t="inlineStr">
@@ -2214,22 +2210,23 @@
       </c>
       <c r="D42" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra đổi Tỉnh/Thành phố reload các trường phụ thuộc</t>
+          <t>Kiểm tra tìm kiếm và chọn Phường/Xã</t>
         </is>
       </c>
       <c r="E42" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 Tỉnh/Thành phố</t>
+          <t>- Đã chọn Tỉnh/Thành phố</t>
         </is>
       </c>
       <c r="F42" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn 1 Tỉnh/Thành phố khác</t>
+          <t>1. Tìm Phường/Xã theo tên
+2. Chọn 1 Phường/Xã</t>
         </is>
       </c>
       <c r="G42" s="41" t="inlineStr">
         <is>
-          <t>Reload Phường/Xã tương ứng, reset Tên đường, trigger kiểm tra chính sách giá</t>
+          <t>Hiển thị danh sách khớp; chỉ chọn được 1 và hiển thị đúng giá trị</t>
         </is>
       </c>
       <c r="H42" s="40" t="inlineStr">
@@ -2254,28 +2251,28 @@
       </c>
       <c r="C43" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D43" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra pre-fill "Địa chỉ trước sáp nhập" điền toàn bộ địa chỉ</t>
+          <t>Kiểm tra đổi Phường/Xã gọi API chính sách kiểm tra lại giá</t>
         </is>
       </c>
       <c r="E43" s="41" t="inlineStr">
         <is>
-          <t>- Account đã có địa chỉ lưu sẵn từ đơn trước
-- Dịch vụ có link "Địa chỉ trước sáp nhập"</t>
+          <t>- Đã chọn Tỉnh/Thành phố và Phường/Xã</t>
         </is>
       </c>
       <c r="F43" s="41" t="inlineStr">
         <is>
-          <t>1. Click link "Địa chỉ trước sáp nhập"</t>
+          <t>1. Đổi sang Phường/Xã khác
+2. Quan sát Tạm tính/Giá</t>
         </is>
       </c>
       <c r="G43" s="41" t="inlineStr">
         <is>
-          <t>Hệ thống tự điền TOÀN BỘ địa chỉ đã lưu (Tỉnh/TP, Phường/Xã, Tên đường, Số nhà...)</t>
+          <t>Reset Tên đường; gọi API chính sách: giá không đổi → giữ Tạm tính; giá đổi → cập nhật lại Tạm tính</t>
         </is>
       </c>
       <c r="H43" s="40" t="inlineStr">
@@ -2289,21 +2286,51 @@
       <c r="L43" s="42" t="n"/>
     </row>
     <row r="44" ht="15" customHeight="1" s="32">
-      <c r="B44" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 7: Block Địa chỉ lắp đặt — Phường/Xã &amp; kiểm tra chính sách giá</t>
-        </is>
-      </c>
-      <c r="C44" s="35" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="35" t="n"/>
-      <c r="F44" s="35" t="n"/>
-      <c r="G44" s="35" t="n"/>
-      <c r="H44" s="35" t="n"/>
-      <c r="I44" s="35" t="n"/>
-      <c r="J44" s="35" t="n"/>
-      <c r="K44" s="35" t="n"/>
-      <c r="L44" s="36" t="n"/>
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B44" s="40">
+        <f>IF(D44="","",$D$3&amp;"."&amp;COUNTA($D$10:D44)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C44" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D44" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn địa chỉ không có chính sách hiển thị popup "Chưa hỗ trợ chính sách!"</t>
+        </is>
+      </c>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
+        </is>
+      </c>
+      <c r="F44" s="41" t="inlineStr">
+        <is>
+          <t>1. Chọn Tỉnh/Phường-Xã không có chính sách
+2. Quan sát popup
+3. Click btn Đóng</t>
+        </is>
+      </c>
+      <c r="G44" s="41" t="inlineStr">
+        <is>
+          <t>[BLOCKED – cần confirm nội dung đầy đủ popup (CLA-CKCOMMON-007 BA bổ sung sau)]. Theo rule (Rule common R5): hiển thị popup "Chưa hỗ trợ chính sách!" → đồng thời đẩy KHTN → tắt thông báo và quay về homepage (KHÔNG cho qua bước thanh toán)</t>
+        </is>
+      </c>
+      <c r="H44" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I44" s="42" t="n"/>
+      <c r="J44" s="42" t="n"/>
+      <c r="K44" s="42" t="n"/>
+      <c r="L44" s="42" t="n"/>
     </row>
     <row r="45" ht="28.35" customHeight="1" s="32">
       <c r="A45" s="39" t="inlineStr">
@@ -2322,28 +2349,29 @@
       </c>
       <c r="D45" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Phường/Xã placeholder và bắt buộc chọn</t>
+          <t>Kiểm tra đẩy KHTN khi chọn địa chỉ không có chính sách</t>
         </is>
       </c>
       <c r="E45" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn Tỉnh/Thành phố</t>
+          <t>- Đã chọn địa chỉ không có chính sách
+- Có thể đẩy KHTN thành công</t>
         </is>
       </c>
       <c r="F45" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát placeholder Phường/Xã
-2. Không chọn và click ra ngoài</t>
+          <t>1. Đóng popup Chưa hỗ trợ chính sách
+2. Truy cập web-admin (saleplatform-stag) kiểm tra KHTN theo SĐT đã nhập</t>
         </is>
       </c>
       <c r="G45" s="41" t="inlineStr">
         <is>
-          <t>Placeholder "Chọn phường/xã"; border đỏ + "Vui lòng chọn phường/xã."</t>
+          <t>Đẩy KHTN thành công tương ứng SĐT đã nhập</t>
         </is>
       </c>
       <c r="H45" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I45" s="42" t="n"/>
@@ -2352,50 +2380,21 @@
       <c r="L45" s="42" t="n"/>
     </row>
     <row r="46" ht="28.35" customHeight="1" s="32">
-      <c r="A46" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B46" s="40">
-        <f>IF(D46="","",$D$3&amp;"."&amp;COUNTA($D$10:D46)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C46" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D46" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra tìm kiếm và chọn Phường/Xã</t>
-        </is>
-      </c>
-      <c r="E46" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn Tỉnh/Thành phố</t>
-        </is>
-      </c>
-      <c r="F46" s="41" t="inlineStr">
-        <is>
-          <t>1. Tìm Phường/Xã theo tên
-2. Chọn 1 Phường/Xã</t>
-        </is>
-      </c>
-      <c r="G46" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị danh sách khớp; chỉ chọn được 1 và hiển thị đúng giá trị</t>
-        </is>
-      </c>
-      <c r="H46" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I46" s="42" t="n"/>
-      <c r="J46" s="42" t="n"/>
-      <c r="K46" s="42" t="n"/>
-      <c r="L46" s="42" t="n"/>
+      <c r="B46" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 7: Block Địa chỉ lắp đặt — Tên đường</t>
+        </is>
+      </c>
+      <c r="C46" s="35" t="n"/>
+      <c r="D46" s="35" t="n"/>
+      <c r="E46" s="35" t="n"/>
+      <c r="F46" s="35" t="n"/>
+      <c r="G46" s="35" t="n"/>
+      <c r="H46" s="35" t="n"/>
+      <c r="I46" s="35" t="n"/>
+      <c r="J46" s="35" t="n"/>
+      <c r="K46" s="35" t="n"/>
+      <c r="L46" s="36" t="n"/>
     </row>
     <row r="47" ht="28.35" customHeight="1" s="32">
       <c r="A47" s="39" t="inlineStr">
@@ -2409,28 +2408,28 @@
       </c>
       <c r="C47" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D47" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra đổi Phường/Xã gọi API chính sách kiểm tra lại giá</t>
+          <t>Kiểm tra Tên đường placeholder và bắt buộc chọn</t>
         </is>
       </c>
       <c r="E47" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn Tỉnh/Thành phố và Phường/Xã</t>
+          <t>- Đã chọn Phường/Xã</t>
         </is>
       </c>
       <c r="F47" s="41" t="inlineStr">
         <is>
-          <t>1. Đổi sang Phường/Xã khác
-2. Quan sát Tạm tính/Giá</t>
+          <t>1. Quan sát placeholder Tên đường
+2. Không chọn và click ra ngoài</t>
         </is>
       </c>
       <c r="G47" s="41" t="inlineStr">
         <is>
-          <t>Reset Tên đường; gọi API chính sách: giá không đổi → giữ Tạm tính; giá đổi → cập nhật lại Tạm tính</t>
+          <t>Placeholder "Chọn tên đường"; border đỏ + "Vui lòng chọn tên đường."</t>
         </is>
       </c>
       <c r="H47" s="40" t="inlineStr">
@@ -2455,29 +2454,28 @@
       </c>
       <c r="C48" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D48" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra chọn địa chỉ không có chính sách hiển thị popup "Chưa hỗ trợ chính sách!"</t>
+          <t>Kiểm tra tìm kiếm và chọn Tên đường</t>
         </is>
       </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
+          <t>- Đã chọn Phường/Xã</t>
         </is>
       </c>
       <c r="F48" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn Tỉnh/Phường-Xã không có chính sách
-2. Quan sát popup
-3. Click btn Đóng</t>
+          <t>1. Nhập từ khóa tìm Tên đường
+2. Chọn 1 Tên đường</t>
         </is>
       </c>
       <c r="G48" s="41" t="inlineStr">
         <is>
-          <t>[BLOCKED – cần confirm nội dung đầy đủ popup (CLA-CKCOMMON-007 BA bổ sung sau)]. Theo rule (Rule common R5): hiển thị popup "Chưa hỗ trợ chính sách!" → đồng thời đẩy KHTN → tắt thông báo và quay về homepage (KHÔNG cho qua bước thanh toán)</t>
+          <t>Tìm theo quy tắc contains, không trim khoảng trắng trước khi tìm; chỉ chọn được 1</t>
         </is>
       </c>
       <c r="H48" s="40" t="inlineStr">
@@ -2491,68 +2489,67 @@
       <c r="L48" s="42" t="n"/>
     </row>
     <row r="49" ht="41.75" customHeight="1" s="32">
-      <c r="A49" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B49" s="40">
-        <f>IF(D49="","",$D$3&amp;"."&amp;COUNTA($D$10:D49)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C49" s="40" t="inlineStr">
+      <c r="B49" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 8: Block Địa chỉ lắp đặt — Số nhà (radio Nhà riêng/Chung cư: đặc thù dịch vụ thiết bị; Chung cư DEFERRED)</t>
+        </is>
+      </c>
+      <c r="C49" s="35" t="n"/>
+      <c r="D49" s="35" t="n"/>
+      <c r="E49" s="35" t="n"/>
+      <c r="F49" s="35" t="n"/>
+      <c r="G49" s="35" t="n"/>
+      <c r="H49" s="35" t="n"/>
+      <c r="I49" s="35" t="n"/>
+      <c r="J49" s="35" t="n"/>
+      <c r="K49" s="35" t="n"/>
+      <c r="L49" s="36" t="n"/>
+    </row>
+    <row r="50" ht="15" customHeight="1" s="32">
+      <c r="A50" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B50" s="40">
+        <f>IF(D50="","",$D$3&amp;"."&amp;COUNTA($D$10:D50)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C50" s="40" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="D49" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra đẩy KHTN khi chọn địa chỉ không có chính sách</t>
-        </is>
-      </c>
-      <c r="E49" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn địa chỉ không có chính sách
-- Có thể đẩy KHTN thành công</t>
-        </is>
-      </c>
-      <c r="F49" s="41" t="inlineStr">
-        <is>
-          <t>1. Đóng popup Chưa hỗ trợ chính sách
-2. Truy cập web-admin (saleplatform-stag) kiểm tra KHTN theo SĐT đã nhập</t>
-        </is>
-      </c>
-      <c r="G49" s="41" t="inlineStr">
-        <is>
-          <t>Đẩy KHTN thành công tương ứng SĐT đã nhập</t>
-        </is>
-      </c>
-      <c r="H49" s="40" t="inlineStr">
+      <c r="D50" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra radio Nhà riêng/Chung cư (đặc thù dịch vụ thiết bị)</t>
+        </is>
+      </c>
+      <c r="E50" s="41" t="inlineStr">
+        <is>
+          <t>- Block Địa chỉ lắp đặt đang hiển thị
+- Dịch vụ thiết bị (VD Camera) — Rule common không định nghĩa radio này</t>
+        </is>
+      </c>
+      <c r="F50" s="41" t="inlineStr">
+        <is>
+          <t>1. Quan sát Block Địa chỉ lắp đặt</t>
+        </is>
+      </c>
+      <c r="G50" s="41" t="inlineStr">
+        <is>
+          <t>Rule common KHÔNG có radio Nhà riêng/Chung cư. Tất cả dịch vụ chỉ có trường Số nhà, không hiển thi 2 radio Nhà riêng, Chung cư</t>
+        </is>
+      </c>
+      <c r="H50" s="40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I49" s="42" t="n"/>
-      <c r="J49" s="42" t="n"/>
-      <c r="K49" s="42" t="n"/>
-      <c r="L49" s="42" t="n"/>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="32">
-      <c r="B50" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 8: Block Địa chỉ lắp đặt — Tên đường</t>
-        </is>
-      </c>
-      <c r="C50" s="35" t="n"/>
-      <c r="D50" s="35" t="n"/>
-      <c r="E50" s="35" t="n"/>
-      <c r="F50" s="35" t="n"/>
-      <c r="G50" s="35" t="n"/>
-      <c r="H50" s="35" t="n"/>
-      <c r="I50" s="35" t="n"/>
-      <c r="J50" s="35" t="n"/>
-      <c r="K50" s="35" t="n"/>
-      <c r="L50" s="36" t="n"/>
+      <c r="I50" s="42" t="n"/>
+      <c r="J50" s="42" t="n"/>
+      <c r="K50" s="42" t="n"/>
+      <c r="L50" s="42" t="n"/>
     </row>
     <row r="51" ht="28.35" customHeight="1" s="32">
       <c r="A51" s="39" t="inlineStr">
@@ -2571,23 +2568,22 @@
       </c>
       <c r="D51" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Tên đường placeholder và bắt buộc chọn</t>
+          <t>Kiểm tra Số nhà để trống → báo lỗi bắt buộc</t>
         </is>
       </c>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn Phường/Xã</t>
+          <t>- Đã chọn đủ Tỉnh/Phường-Xã/Tên đường (trường Số nhà* đang hiển thị)</t>
         </is>
       </c>
       <c r="F51" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát placeholder Tên đường
-2. Không chọn và click ra ngoài</t>
+          <t>1. Để trống Số nhà và click ra ngoài / submit</t>
         </is>
       </c>
       <c r="G51" s="41" t="inlineStr">
         <is>
-          <t>Placeholder "Chọn tên đường"; border đỏ + "Vui lòng chọn tên đường."</t>
+          <t>Border đỏ và hiển thị "Vui lòng nhập số nhà."</t>
         </is>
       </c>
       <c r="H51" s="40" t="inlineStr">
@@ -2617,23 +2613,22 @@
       </c>
       <c r="D52" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra tìm kiếm và chọn Tên đường</t>
+          <t>Kiểm tra Số nhà nhập/paste vượt quá 50 ký tự</t>
         </is>
       </c>
       <c r="E52" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn Phường/Xã</t>
+          <t>- Trường Số nhà* đang hiển thị</t>
         </is>
       </c>
       <c r="F52" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập từ khóa tìm Tên đường
-2. Chọn 1 Tên đường</t>
+          <t>1. Nhập/paste Số nhà dài hơn 50 ký tự</t>
         </is>
       </c>
       <c r="G52" s="41" t="inlineStr">
         <is>
-          <t>Tìm theo quy tắc contains, không trim khoảng trắng trước khi tìm; chỉ chọn được 1</t>
+          <t>Chỉ cho nhập và hiển thị tối đa 50 ký tự</t>
         </is>
       </c>
       <c r="H52" s="40" t="inlineStr">
@@ -2649,7 +2644,7 @@
     <row r="53" ht="15" customHeight="1" s="32">
       <c r="B53" s="38" t="inlineStr">
         <is>
-          <t>Nhóm 9: Block Địa chỉ lắp đặt — Số nhà (radio Nhà riêng/Chung cư: đặc thù dịch vụ thiết bị; Chung cư DEFERRED)</t>
+          <t>Nhóm 9: Block Địa chỉ lắp đặt — Ghi chú</t>
         </is>
       </c>
       <c r="C53" s="35" t="n"/>
@@ -2675,33 +2670,34 @@
       </c>
       <c r="C54" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D54" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra radio Nhà riêng/Chung cư (đặc thù dịch vụ thiết bị)</t>
+          <t>Kiểm tra Ghi chú placeholder, không bắt buộc và giới hạn 100 ký tự</t>
         </is>
       </c>
       <c r="E54" s="41" t="inlineStr">
         <is>
-          <t>- Block Địa chỉ lắp đặt đang hiển thị
-- Dịch vụ thiết bị (VD Camera) — Rule common không định nghĩa radio này</t>
+          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
         </is>
       </c>
       <c r="F54" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát Block Địa chỉ lắp đặt</t>
+          <t>1. Quan sát placeholder Ghi chú
+2. Để trống rồi click ra ngoài
+3. Nhập/paste &gt; 100 ký tự</t>
         </is>
       </c>
       <c r="G54" s="41" t="inlineStr">
         <is>
-          <t>Rule common KHÔNG có radio Nhà riêng/Chung cư. Tất cả dịch vụ chỉ có trường Số nhà, không hiển thi 2 radio Nhà riêng, Chung cư</t>
+          <t>Placeholder "Gọi cho tôi trước 30 phút nhé!"; để trống không báo lỗi; nhập &gt; 100 → chỉ nhận 100 ký tự</t>
         </is>
       </c>
       <c r="H54" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I54" s="42" t="n"/>
@@ -2710,49 +2706,21 @@
       <c r="L54" s="42" t="n"/>
     </row>
     <row r="55" ht="28.35" customHeight="1" s="32">
-      <c r="A55" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B55" s="40">
-        <f>IF(D55="","",$D$3&amp;"."&amp;COUNTA($D$10:D55)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C55" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D55" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra Số nhà để trống → báo lỗi bắt buộc</t>
-        </is>
-      </c>
-      <c r="E55" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn đủ Tỉnh/Phường-Xã/Tên đường (trường Số nhà* đang hiển thị)</t>
-        </is>
-      </c>
-      <c r="F55" s="41" t="inlineStr">
-        <is>
-          <t>1. Để trống Số nhà và click ra ngoài / submit</t>
-        </is>
-      </c>
-      <c r="G55" s="41" t="inlineStr">
-        <is>
-          <t>Border đỏ và hiển thị "Vui lòng nhập số nhà."</t>
-        </is>
-      </c>
-      <c r="H55" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I55" s="42" t="n"/>
-      <c r="J55" s="42" t="n"/>
-      <c r="K55" s="42" t="n"/>
-      <c r="L55" s="42" t="n"/>
+      <c r="B55" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 10: Popup Địa chỉ hành chính cũ (3 cấp → 2 cấp)</t>
+        </is>
+      </c>
+      <c r="C55" s="35" t="n"/>
+      <c r="D55" s="35" t="n"/>
+      <c r="E55" s="35" t="n"/>
+      <c r="F55" s="35" t="n"/>
+      <c r="G55" s="35" t="n"/>
+      <c r="H55" s="35" t="n"/>
+      <c r="I55" s="35" t="n"/>
+      <c r="J55" s="35" t="n"/>
+      <c r="K55" s="35" t="n"/>
+      <c r="L55" s="36" t="n"/>
     </row>
     <row r="56" ht="28.35" customHeight="1" s="32">
       <c r="A56" s="39" t="inlineStr">
@@ -2771,22 +2739,22 @@
       </c>
       <c r="D56" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Số nhà nhập/paste vượt quá 50 ký tự</t>
+          <t>Kiểm tra hiển thị UI popup Địa chỉ hành chính cũ</t>
         </is>
       </c>
       <c r="E56" s="41" t="inlineStr">
         <is>
-          <t>- Trường Số nhà* đang hiển thị</t>
+          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
         </is>
       </c>
       <c r="F56" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập/paste Số nhà dài hơn 50 ký tự</t>
+          <t>1. Click link "Địa chỉ trước sáp nhập"</t>
         </is>
       </c>
       <c r="G56" s="41" t="inlineStr">
         <is>
-          <t>Chỉ cho nhập và hiển thị tối đa 50 ký tự</t>
+          <t>Popup hiển thị: title "Địa chỉ hành chính cũ", label hướng dẫn, 4 dropdown (Tỉnh/TP, Quận/Huyện, Phường/Xã, Tên đường), icon X, button Xác nhận</t>
         </is>
       </c>
       <c r="H56" s="40" t="inlineStr">
@@ -2800,21 +2768,50 @@
       <c r="L56" s="42" t="n"/>
     </row>
     <row r="57" ht="15" customHeight="1" s="32">
-      <c r="B57" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 10: Block Địa chỉ lắp đặt — Ghi chú</t>
-        </is>
-      </c>
-      <c r="C57" s="35" t="n"/>
-      <c r="D57" s="35" t="n"/>
-      <c r="E57" s="35" t="n"/>
-      <c r="F57" s="35" t="n"/>
-      <c r="G57" s="35" t="n"/>
-      <c r="H57" s="35" t="n"/>
-      <c r="I57" s="35" t="n"/>
-      <c r="J57" s="35" t="n"/>
-      <c r="K57" s="35" t="n"/>
-      <c r="L57" s="36" t="n"/>
+      <c r="A57" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B57" s="40">
+        <f>IF(D57="","",$D$3&amp;"."&amp;COUNTA($D$10:D57)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D57" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra load phân cấp và tìm kiếm trong popup Địa chỉ hành chính cũ</t>
+        </is>
+      </c>
+      <c r="E57" s="41" t="inlineStr">
+        <is>
+          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
+        </is>
+      </c>
+      <c r="F57" s="41" t="inlineStr">
+        <is>
+          <t>1. Chọn Tỉnh/TP → Quận/Huyện → Phường/Xã → Tên đường
+2. Tìm kiếm ở từng cấp</t>
+        </is>
+      </c>
+      <c r="G57" s="41" t="inlineStr">
+        <is>
+          <t>63 tỉnh theo ĐCHC 3 cấp; mỗi cấp load theo cấp trên; tìm kiếm contains, không trim</t>
+        </is>
+      </c>
+      <c r="H57" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I57" s="42" t="n"/>
+      <c r="J57" s="42" t="n"/>
+      <c r="K57" s="42" t="n"/>
+      <c r="L57" s="42" t="n"/>
     </row>
     <row r="58" ht="41.75" customHeight="1" s="32">
       <c r="A58" s="39" t="inlineStr">
@@ -2828,29 +2825,28 @@
       </c>
       <c r="C58" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D58" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra Ghi chú placeholder, không bắt buộc và giới hạn 100 ký tự</t>
+          <t>Kiểm tra button Xác nhận disable khi chưa chọn đủ 4 cấp</t>
         </is>
       </c>
       <c r="E58" s="41" t="inlineStr">
         <is>
-          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
+          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
         </is>
       </c>
       <c r="F58" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát placeholder Ghi chú
-2. Để trống rồi click ra ngoài
-3. Nhập/paste &gt; 100 ký tự</t>
+          <t>1. Để trống bất kỳ 1 trong 4 cấp
+2. Quan sát button Xác nhận</t>
         </is>
       </c>
       <c r="G58" s="41" t="inlineStr">
         <is>
-          <t>Placeholder "Gọi cho tôi trước 30 phút nhé!"; để trống không báo lỗi; nhập &gt; 100 → chỉ nhận 100 ký tự</t>
+          <t>Button Xác nhận ở trạng thái disable</t>
         </is>
       </c>
       <c r="H58" s="40" t="inlineStr">
@@ -2864,55 +2860,81 @@
       <c r="L58" s="42" t="n"/>
     </row>
     <row r="59" ht="15" customHeight="1" s="32">
-      <c r="B59" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 11: Popup Địa chỉ hành chính cũ (3 cấp → 2 cấp)</t>
-        </is>
-      </c>
-      <c r="C59" s="35" t="n"/>
-      <c r="D59" s="35" t="n"/>
-      <c r="E59" s="35" t="n"/>
-      <c r="F59" s="35" t="n"/>
-      <c r="G59" s="35" t="n"/>
-      <c r="H59" s="35" t="n"/>
-      <c r="I59" s="35" t="n"/>
-      <c r="J59" s="35" t="n"/>
-      <c r="K59" s="35" t="n"/>
-      <c r="L59" s="36" t="n"/>
+      <c r="A59" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B59" s="40">
+        <f>IF(D59="","",$D$3&amp;"."&amp;COUNTA($D$10:D59)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D59" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra chọn đủ 4 cấp hiển thị Địa chỉ hành chính mới và enable Xác nhận</t>
+        </is>
+      </c>
+      <c r="E59" s="41" t="inlineStr">
+        <is>
+          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
+        </is>
+      </c>
+      <c r="F59" s="41" t="inlineStr">
+        <is>
+          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường</t>
+        </is>
+      </c>
+      <c r="G59" s="41" t="inlineStr">
+        <is>
+          <t>Hiển thị field "Địa chỉ hành chính mới" (convert 3 cấp → 2 cấp); &lt;giá trị khi convert thành công&gt;
+→ data test tôi sẽ cung cấp lại sau</t>
+        </is>
+      </c>
+      <c r="H59" s="40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I59" s="42" t="n"/>
+      <c r="J59" s="42" t="n"/>
+      <c r="K59" s="42" t="n"/>
+      <c r="L59" s="42" t="n"/>
     </row>
     <row r="60" ht="41.75" customHeight="1" s="32">
-      <c r="A60" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
+      <c r="A60" s="39" t="n"/>
       <c r="B60" s="40">
         <f>IF(D60="","",$D$3&amp;"."&amp;COUNTA($D$10:D60)&amp;"")</f>
         <v/>
       </c>
       <c r="C60" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D60" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hiển thị UI popup Địa chỉ hành chính cũ</t>
+          <t xml:space="preserve">Kiểm tra btn Xác nhận khi convert địa chỉ từ 3 → 2 cấp thành công </t>
         </is>
       </c>
       <c r="E60" s="41" t="inlineStr">
         <is>
-          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
+          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
         </is>
       </c>
       <c r="F60" s="41" t="inlineStr">
         <is>
-          <t>1. Click link "Địa chỉ trước sáp nhập"</t>
+          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường có data convert hợp lệ
+2. Quan sát btn Xác nhận</t>
         </is>
       </c>
       <c r="G60" s="41" t="inlineStr">
         <is>
-          <t>Popup hiển thị: title "Địa chỉ hành chính cũ", label hướng dẫn, 4 dropdown (Tỉnh/TP, Quận/Huyện, Phường/Xã, Tên đường), icon X, button Xác nhận</t>
+          <t>Button Xác nhận ở trạng thái Enable</t>
         </is>
       </c>
       <c r="H60" s="40" t="inlineStr">
@@ -2926,23 +2948,19 @@
       <c r="L60" s="42" t="n"/>
     </row>
     <row r="61" ht="41.75" customHeight="1" s="32">
-      <c r="A61" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
+      <c r="A61" s="39" t="n"/>
       <c r="B61" s="40">
         <f>IF(D61="","",$D$3&amp;"."&amp;COUNTA($D$10:D61)&amp;"")</f>
         <v/>
       </c>
       <c r="C61" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D61" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra load phân cấp và tìm kiếm trong popup Địa chỉ hành chính cũ</t>
+          <t xml:space="preserve">Kiểm tra btn Xác nhận khi convert địa chỉ từ 3 → 2 cấp không thành công </t>
         </is>
       </c>
       <c r="E61" s="41" t="inlineStr">
@@ -2952,13 +2970,13 @@
       </c>
       <c r="F61" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn Tỉnh/TP → Quận/Huyện → Phường/Xã → Tên đường
-2. Tìm kiếm ở từng cấp</t>
+          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường có data convert không hợp lệ
+2. Quan sát btn Xác nhận</t>
         </is>
       </c>
       <c r="G61" s="41" t="inlineStr">
         <is>
-          <t>63 tỉnh theo ĐCHC 3 cấp; mỗi cấp load theo cấp trên; tìm kiếm contains, không trim</t>
+          <t>Button Xác nhận ở trạng thái disable</t>
         </is>
       </c>
       <c r="H61" s="40" t="inlineStr">
@@ -2988,23 +3006,22 @@
       </c>
       <c r="D62" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra button Xác nhận disable khi chưa chọn đủ 4 cấp</t>
+          <t>Kiểm tra click icon X đóng popup không cập nhật địa chỉ</t>
         </is>
       </c>
       <c r="E62" s="41" t="inlineStr">
         <is>
-          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
+          <t>- Popup có dữ liệu đã chọn</t>
         </is>
       </c>
       <c r="F62" s="41" t="inlineStr">
         <is>
-          <t>1. Để trống bất kỳ 1 trong 4 cấp
-2. Quan sát button Xác nhận</t>
+          <t>1. Click icon X trên popup</t>
         </is>
       </c>
       <c r="G62" s="41" t="inlineStr">
         <is>
-          <t>Button Xác nhận ở trạng thái disable</t>
+          <t>Không cập nhật địa chỉ mới; đóng popup, về form đăng ký</t>
         </is>
       </c>
       <c r="H62" s="40" t="inlineStr">
@@ -3034,28 +3051,27 @@
       </c>
       <c r="D63" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra chọn đủ 4 cấp hiển thị Địa chỉ hành chính mới và enable Xác nhận</t>
+          <t>Kiểm tra click Xác nhận đẩy địa chỉ 2 cấp vào form</t>
         </is>
       </c>
       <c r="E63" s="41" t="inlineStr">
         <is>
-          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
+          <t>- Popup đã chọn đủ 4 cấp, button Xác nhận enable</t>
         </is>
       </c>
       <c r="F63" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường</t>
+          <t>1. Click button Xác nhận</t>
         </is>
       </c>
       <c r="G63" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị field "Địa chỉ hành chính mới" (convert 3 cấp → 2 cấp); &lt;giá trị khi convert thành công&gt;
-→ data test tôi sẽ cung cấp lại sau</t>
+          <t>Đẩy Tỉnh/TP, Phường/Xã, Tên đường (2 cấp) vào dropdown form đăng ký; đóng popup</t>
         </is>
       </c>
       <c r="H63" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I63" s="42" t="n"/>
@@ -3064,77 +3080,56 @@
       <c r="L63" s="42" t="n"/>
     </row>
     <row r="64" ht="39.3" customHeight="1" s="32">
-      <c r="A64" s="39" t="n"/>
-      <c r="B64" s="40">
-        <f>IF(D64="","",$D$3&amp;"."&amp;COUNTA($D$10:D64)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C64" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D64" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kiểm tra btn Xác nhận khi convert địa chỉ từ 3 → 2 cấp thành công </t>
-        </is>
-      </c>
-      <c r="E64" s="41" t="inlineStr">
-        <is>
-          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
-        </is>
-      </c>
-      <c r="F64" s="41" t="inlineStr">
-        <is>
-          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường có data convert hợp lệ
-2. Quan sát btn Xác nhận</t>
-        </is>
-      </c>
-      <c r="G64" s="41" t="inlineStr">
-        <is>
-          <t>Button Xác nhận ở trạng thái Enable</t>
-        </is>
-      </c>
-      <c r="H64" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I64" s="42" t="n"/>
-      <c r="J64" s="42" t="n"/>
-      <c r="K64" s="42" t="n"/>
-      <c r="L64" s="42" t="n"/>
+      <c r="B64" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 11: Block Thông tin khách hàng</t>
+        </is>
+      </c>
+      <c r="C64" s="35" t="n"/>
+      <c r="D64" s="35" t="n"/>
+      <c r="E64" s="35" t="n"/>
+      <c r="F64" s="35" t="n"/>
+      <c r="G64" s="35" t="n"/>
+      <c r="H64" s="35" t="n"/>
+      <c r="I64" s="35" t="n"/>
+      <c r="J64" s="35" t="n"/>
+      <c r="K64" s="35" t="n"/>
+      <c r="L64" s="36" t="n"/>
     </row>
     <row r="65" ht="39.3" customHeight="1" s="32">
-      <c r="A65" s="39" t="n"/>
+      <c r="A65" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
       <c r="B65" s="40">
         <f>IF(D65="","",$D$3&amp;"."&amp;COUNTA($D$10:D65)&amp;"")</f>
         <v/>
       </c>
       <c r="C65" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D65" s="41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiểm tra btn Xác nhận khi convert địa chỉ từ 3 → 2 cấp không thành công </t>
+          <t>Kiểm tra thu gọn/mở rộng block Thông tin khách hàng</t>
         </is>
       </c>
       <c r="E65" s="41" t="inlineStr">
         <is>
-          <t>- Popup Địa chỉ hành chính cũ đang mở</t>
+          <t>- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F65" s="41" t="inlineStr">
         <is>
-          <t>1. Chọn đủ Tỉnh/TP + Quận/Huyện + Phường/Xã + Tên đường có data convert không hợp lệ
-2. Quan sát btn Xác nhận</t>
+          <t>1. Click icon Collapse
+2. Click icon Expand</t>
         </is>
       </c>
       <c r="G65" s="41" t="inlineStr">
         <is>
-          <t>Button Xác nhận ở trạng thái disable</t>
+          <t>Thu gọn/mở rộng các trường; icon đổi collapse ↔ expand</t>
         </is>
       </c>
       <c r="H65" s="40" t="inlineStr">
@@ -3164,22 +3159,22 @@
       </c>
       <c r="D66" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click icon X đóng popup không cập nhật địa chỉ</t>
+          <t>Kiểm tra format hiển thị địa chỉ Nhà riêng trong block Thông tin khách hàng</t>
         </is>
       </c>
       <c r="E66" s="41" t="inlineStr">
         <is>
-          <t>- Popup có dữ liệu đã chọn</t>
+          <t>- Đã nhập đủ địa chỉ loại Nhà riêng</t>
         </is>
       </c>
       <c r="F66" s="41" t="inlineStr">
         <is>
-          <t>1. Click icon X trên popup</t>
+          <t>1. Quan sát địa chỉ trong block Thông tin khách hàng</t>
         </is>
       </c>
       <c r="G66" s="41" t="inlineStr">
         <is>
-          <t>Không cập nhật địa chỉ mới; đóng popup, về form đăng ký</t>
+          <t>Hiển thị theo format: Số nhà, Tên đường, Phường/Xã, Tỉnh/Thành</t>
         </is>
       </c>
       <c r="H66" s="40" t="inlineStr">
@@ -3204,27 +3199,27 @@
       </c>
       <c r="C67" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D67" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click Xác nhận đẩy địa chỉ 2 cấp vào form</t>
+          <t>Kiểm tra không cho chỉnh sửa thông tin trong block Thông tin khách hàng</t>
         </is>
       </c>
       <c r="E67" s="41" t="inlineStr">
         <is>
-          <t>- Popup đã chọn đủ 4 cấp, button Xác nhận enable</t>
+          <t>- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F67" s="41" t="inlineStr">
         <is>
-          <t>1. Click button Xác nhận</t>
+          <t>1. Cố chỉnh sửa Họ tên/SĐT/Email/Địa chỉ trong block Thông tin khách hàng</t>
         </is>
       </c>
       <c r="G67" s="41" t="inlineStr">
         <is>
-          <t>Đẩy Tỉnh/TP, Phường/Xã, Tên đường (2 cấp) vào dropdown form đăng ký; đóng popup</t>
+          <t>Không thể chỉnh sửa (read-only)</t>
         </is>
       </c>
       <c r="H67" s="40" t="inlineStr">
@@ -3240,7 +3235,7 @@
     <row r="68" ht="15" customHeight="1" s="32">
       <c r="B68" s="38" t="inlineStr">
         <is>
-          <t>Nhóm 12: Block Thông tin khách hàng</t>
+          <t>Nhóm 12: Block Phương thức thanh toán</t>
         </is>
       </c>
       <c r="C68" s="35" t="n"/>
@@ -3266,28 +3261,27 @@
       </c>
       <c r="C69" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D69" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra thu gọn/mở rộng block Thông tin khách hàng</t>
+          <t>Kiểm tra hiển thị UI block Phương thức thanh toán</t>
         </is>
       </c>
       <c r="E69" s="41" t="inlineStr">
         <is>
-          <t>- Đang ở màn hình Checkout</t>
+          <t>- Dịch vụ có ít nhất 1 PTTT trong chính sách</t>
         </is>
       </c>
       <c r="F69" s="41" t="inlineStr">
         <is>
-          <t>1. Click icon Collapse
-2. Click icon Expand</t>
+          <t>1. Quan sát block Phương thức thanh toán</t>
         </is>
       </c>
       <c r="G69" s="41" t="inlineStr">
         <is>
-          <t>Thu gọn/mở rộng các trường; icon đổi collapse ↔ expand</t>
+          <t>Hiển thị: radio chọn, icon PTTT, tên PTTT, miêu tả, số lượng ưu đãi, button Xem thêm/Rút gọn (tùy số PTTT)</t>
         </is>
       </c>
       <c r="H69" s="40" t="inlineStr">
@@ -3312,32 +3306,32 @@
       </c>
       <c r="C70" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D70" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra format hiển thị địa chỉ Nhà riêng trong block Thông tin khách hàng</t>
+          <t>Kiểm tra hiển thị khi chính sách có ≤ 4 PTTT</t>
         </is>
       </c>
       <c r="E70" s="41" t="inlineStr">
         <is>
-          <t>- Đã nhập đủ địa chỉ loại Nhà riêng</t>
+          <t>- Chính sách có dưới 4 PTTT</t>
         </is>
       </c>
       <c r="F70" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát địa chỉ trong block Thông tin khách hàng</t>
+          <t>1. Quan sát block Phương thức thanh toán</t>
         </is>
       </c>
       <c r="G70" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị theo format: Số nhà, Tên đường, Phường/Xã, Tỉnh/Thành</t>
+          <t>Hiển thị tất cả PTTT, không có button Xem thêm</t>
         </is>
       </c>
       <c r="H70" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I70" s="42" t="n"/>
@@ -3357,27 +3351,29 @@
       </c>
       <c r="C71" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D71" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra không cho chỉnh sửa thông tin trong block Thông tin khách hàng</t>
+          <t>Kiểm tra hiển thị và Xem thêm/Thu gọn khi &gt; 4 PTTT</t>
         </is>
       </c>
       <c r="E71" s="41" t="inlineStr">
         <is>
-          <t>- Đang ở màn hình Checkout</t>
+          <t>- Chính sách có hơn 4 PTTT</t>
         </is>
       </c>
       <c r="F71" s="41" t="inlineStr">
         <is>
-          <t>1. Cố chỉnh sửa Họ tên/SĐT/Email/Địa chỉ trong block Thông tin khách hàng</t>
+          <t>1. Quan sát số PTTT hiển thị mặc định
+2. Click Xem thêm
+3. Click Thu gọn</t>
         </is>
       </c>
       <c r="G71" s="41" t="inlineStr">
         <is>
-          <t>Không thể chỉnh sửa (read-only)</t>
+          <t>Mặc định hiển thị 4 PTTT đầu + Xem thêm; Xem thêm → hiển thị hết; Thu gọn → còn 4 PTTT đầu</t>
         </is>
       </c>
       <c r="H71" s="40" t="inlineStr">
@@ -3391,66 +3387,67 @@
       <c r="L71" s="42" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1" s="32">
-      <c r="B72" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 13: Block Phương thức thanh toán</t>
-        </is>
-      </c>
-      <c r="C72" s="35" t="n"/>
-      <c r="D72" s="35" t="n"/>
-      <c r="E72" s="35" t="n"/>
-      <c r="F72" s="35" t="n"/>
-      <c r="G72" s="35" t="n"/>
-      <c r="H72" s="35" t="n"/>
-      <c r="I72" s="35" t="n"/>
-      <c r="J72" s="35" t="n"/>
-      <c r="K72" s="35" t="n"/>
-      <c r="L72" s="36" t="n"/>
+      <c r="A72" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B72" s="40">
+        <f>IF(D72="","",$D$3&amp;"."&amp;COUNTA($D$10:D72)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C72" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D72" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra default option, chỉ chọn 1 và không bỏ chọn được</t>
+        </is>
+      </c>
+      <c r="E72" s="41" t="inlineStr">
+        <is>
+          <t>- Block PTTT đang hiển thị</t>
+        </is>
+      </c>
+      <c r="F72" s="41" t="inlineStr">
+        <is>
+          <t>1. Quan sát option mặc định
+2. Cố chọn nhiều option / bỏ chọn option đầu</t>
+        </is>
+      </c>
+      <c r="G72" s="41" t="inlineStr">
+        <is>
+          <t>Option đầu được chọn mặc định, không bỏ chọn được; chỉ chọn được 1 PTTT tại một thời điểm</t>
+        </is>
+      </c>
+      <c r="H72" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I72" s="42" t="n"/>
+      <c r="J72" s="42" t="n"/>
+      <c r="K72" s="42" t="n"/>
+      <c r="L72" s="42" t="n"/>
     </row>
     <row r="73" ht="28.35" customHeight="1" s="32">
-      <c r="A73" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B73" s="40">
-        <f>IF(D73="","",$D$3&amp;"."&amp;COUNTA($D$10:D73)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C73" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D73" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra hiển thị UI block Phương thức thanh toán</t>
-        </is>
-      </c>
-      <c r="E73" s="41" t="inlineStr">
-        <is>
-          <t>- Dịch vụ có ít nhất 1 PTTT trong chính sách</t>
-        </is>
-      </c>
-      <c r="F73" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát block Phương thức thanh toán</t>
-        </is>
-      </c>
-      <c r="G73" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị: radio chọn, icon PTTT, tên PTTT, miêu tả, số lượng ưu đãi, button Xem thêm/Rút gọn (tùy số PTTT)</t>
-        </is>
-      </c>
-      <c r="H73" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I73" s="42" t="n"/>
-      <c r="J73" s="42" t="n"/>
-      <c r="K73" s="42" t="n"/>
-      <c r="L73" s="42" t="n"/>
+      <c r="B73" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 13: Block Thông tin thanh toán &amp; Mã ưu đãi</t>
+        </is>
+      </c>
+      <c r="C73" s="35" t="n"/>
+      <c r="D73" s="35" t="n"/>
+      <c r="E73" s="35" t="n"/>
+      <c r="F73" s="35" t="n"/>
+      <c r="G73" s="35" t="n"/>
+      <c r="H73" s="35" t="n"/>
+      <c r="I73" s="35" t="n"/>
+      <c r="J73" s="35" t="n"/>
+      <c r="K73" s="35" t="n"/>
+      <c r="L73" s="36" t="n"/>
     </row>
     <row r="74" ht="28.35" customHeight="1" s="32">
       <c r="A74" s="39" t="inlineStr">
@@ -3464,32 +3461,33 @@
       </c>
       <c r="C74" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D74" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hiển thị khi chính sách có ≤ 4 PTTT</t>
+          <t>Kiểm tra thu gọn/mở rộng và hyperlink điều khoản block Thông tin thanh toán</t>
         </is>
       </c>
       <c r="E74" s="41" t="inlineStr">
         <is>
-          <t>- Chính sách có dưới 4 PTTT</t>
+          <t>- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F74" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát block Phương thức thanh toán</t>
+          <t>1. Click Collapse/Expand block Thông tin thanh toán
+2. Click hyperlink điều khoản</t>
         </is>
       </c>
       <c r="G74" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị tất cả PTTT, không có button Xem thêm</t>
+          <t>Thu gọn/mở rộng hoạt động; click điều khoản → màn hình điều khoản FPT Telecom</t>
         </is>
       </c>
       <c r="H74" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I74" s="42" t="n"/>
@@ -3509,29 +3507,27 @@
       </c>
       <c r="C75" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D75" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hiển thị và Xem thêm/Thu gọn khi &gt; 4 PTTT</t>
+          <t>Kiểm tra hiển thị tên gói và giá theo chính sách</t>
         </is>
       </c>
       <c r="E75" s="41" t="inlineStr">
         <is>
-          <t>- Chính sách có hơn 4 PTTT</t>
+          <t>- Có chính sách giá (chung cư/nhà phố)</t>
         </is>
       </c>
       <c r="F75" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát số PTTT hiển thị mặc định
-2. Click Xem thêm
-3. Click Thu gọn</t>
+          <t>1. Quan sát tên gói và giá tại block Thông tin thanh toán</t>
         </is>
       </c>
       <c r="G75" s="41" t="inlineStr">
         <is>
-          <t>Mặc định hiển thị 4 PTTT đầu + Xem thêm; Xem thêm → hiển thị hết; Thu gọn → còn 4 PTTT đầu</t>
+          <t>Tên gói đúng; giá đúng theo chính sách; mặc định hiển thị giá gói 1 tháng</t>
         </is>
       </c>
       <c r="H75" s="40" t="inlineStr">
@@ -3561,33 +3557,34 @@
       </c>
       <c r="D76" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra thứ tự ưu tiên PTTT có CTKM</t>
+          <t>Kiểm tra ô mã khuyến mãi, link Chọn ưu đãi và trạng thái button Áp dụng</t>
         </is>
       </c>
       <c r="E76" s="41" t="inlineStr">
         <is>
-          <t>- Có PTTT kèm chương trình khuyến mãi</t>
+          <t>- Block Thông tin thanh toán đang hiển thị</t>
         </is>
       </c>
       <c r="F76" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát thứ tự các PTTT</t>
+          <t>1. Quan sát ô mã khi rỗng (button Áp dụng)
+2. Nhập 1 ký tự vào ô mã</t>
         </is>
       </c>
       <c r="G76" s="41" t="inlineStr">
         <is>
-          <t>PTTT có CTKM được ưu tiên hiển thị lên trên</t>
-        </is>
-      </c>
-      <c r="H76" s="40" t="n"/>
+          <t>Ô input placeholder "Nhập mã khuyến mãi" + link "Chọn ưu đãi" (badge số) + button Áp dụng: disable khi rỗng, enable khi có ký tự</t>
+        </is>
+      </c>
+      <c r="H76" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="I76" s="42" t="n"/>
       <c r="J76" s="42" t="n"/>
       <c r="K76" s="42" t="n"/>
-      <c r="L76" s="42" t="inlineStr">
-        <is>
-          <t>Bỏ case này giúp tôi</t>
-        </is>
-      </c>
+      <c r="L76" s="42" t="n"/>
     </row>
     <row r="77" ht="28.35" customHeight="1" s="32">
       <c r="A77" s="39" t="inlineStr">
@@ -3601,28 +3598,27 @@
       </c>
       <c r="C77" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D77" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra default option, chỉ chọn 1 và không bỏ chọn được</t>
+          <t>Kiểm tra click link Chọn ưu đãi mở danh sách ưu đãi</t>
         </is>
       </c>
       <c r="E77" s="41" t="inlineStr">
         <is>
-          <t>- Block PTTT đang hiển thị</t>
+          <t>- Có ưu đãi đang hoạt động</t>
         </is>
       </c>
       <c r="F77" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát option mặc định
-2. Cố chọn nhiều option / bỏ chọn option đầu</t>
+          <t>1. Click link "Chọn ưu đãi"</t>
         </is>
       </c>
       <c r="G77" s="41" t="inlineStr">
         <is>
-          <t>Option đầu được chọn mặc định, không bỏ chọn được; chỉ chọn được 1 PTTT tại một thời điểm</t>
+          <t>Hiển thị danh sách ưu đãi khả dụng; badge đúng số lượng ưu đãi</t>
         </is>
       </c>
       <c r="H77" s="40" t="inlineStr">
@@ -3636,21 +3632,51 @@
       <c r="L77" s="42" t="n"/>
     </row>
     <row r="78" ht="15" customHeight="1" s="32">
-      <c r="B78" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 14: Block Thông tin thanh toán &amp; Mã ưu đãi</t>
-        </is>
-      </c>
-      <c r="C78" s="35" t="n"/>
-      <c r="D78" s="35" t="n"/>
-      <c r="E78" s="35" t="n"/>
-      <c r="F78" s="35" t="n"/>
-      <c r="G78" s="35" t="n"/>
-      <c r="H78" s="35" t="n"/>
-      <c r="I78" s="35" t="n"/>
-      <c r="J78" s="35" t="n"/>
-      <c r="K78" s="35" t="n"/>
-      <c r="L78" s="36" t="n"/>
+      <c r="A78" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B78" s="40">
+        <f>IF(D78="","",$D$3&amp;"."&amp;COUNTA($D$10:D78)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C78" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D78" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra áp dụng mã khuyến mãi hợp lệ</t>
+        </is>
+      </c>
+      <c r="E78" s="41" t="inlineStr">
+        <is>
+          <t>- Có mã khuyến mãi hợp lệ đang hoạt động</t>
+        </is>
+      </c>
+      <c r="F78" s="41" t="inlineStr">
+        <is>
+          <t>1. Nhập mã khuyến mãi hợp lệ
+2. Click Áp dụng
+3. Quan sát Cần thanh toán</t>
+        </is>
+      </c>
+      <c r="G78" s="41" t="inlineStr">
+        <is>
+          <t>Hiển thị giá trị giảm; Cần thanh toán = giá gốc − giá trị giảm (cập nhật đúng)</t>
+        </is>
+      </c>
+      <c r="H78" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I78" s="42" t="n"/>
+      <c r="J78" s="42" t="n"/>
+      <c r="K78" s="42" t="n"/>
+      <c r="L78" s="42" t="n"/>
     </row>
     <row r="79" ht="28.35" customHeight="1" s="32">
       <c r="A79" s="39" t="inlineStr">
@@ -3664,28 +3690,28 @@
       </c>
       <c r="C79" s="40" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D79" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra thu gọn/mở rộng và hyperlink điều khoản block Thông tin thanh toán</t>
+          <t>Kiểm tra áp dụng mã khuyến mãi không hợp lệ/hết hạn</t>
         </is>
       </c>
       <c r="E79" s="41" t="inlineStr">
         <is>
-          <t>- Đang ở màn hình Checkout</t>
+          <t>- Mã khuyến mãi không tồn tại hoặc đã hết hạn</t>
         </is>
       </c>
       <c r="F79" s="41" t="inlineStr">
         <is>
-          <t>1. Click Collapse/Expand block Thông tin thanh toán
-2. Click hyperlink điều khoản</t>
+          <t>1. Nhập mã không hợp lệ/hết hạn
+2. Click Áp dụng</t>
         </is>
       </c>
       <c r="G79" s="41" t="inlineStr">
         <is>
-          <t>Thu gọn/mở rộng hoạt động; click điều khoản → màn hình điều khoản FPT Telecom</t>
+          <t>Hiển thị thông báo lỗi (mã không hợp lệ/hết hạn); Cần thanh toán không thay đổi</t>
         </is>
       </c>
       <c r="H79" s="40" t="inlineStr">
@@ -3699,49 +3725,21 @@
       <c r="L79" s="42" t="n"/>
     </row>
     <row r="80" ht="28.35" customHeight="1" s="32">
-      <c r="A80" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B80" s="40">
-        <f>IF(D80="","",$D$3&amp;"."&amp;COUNTA($D$10:D80)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C80" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D80" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra hiển thị tên gói và giá theo chính sách</t>
-        </is>
-      </c>
-      <c r="E80" s="41" t="inlineStr">
-        <is>
-          <t>- Có chính sách giá (chung cư/nhà phố)</t>
-        </is>
-      </c>
-      <c r="F80" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát tên gói và giá tại block Thông tin thanh toán</t>
-        </is>
-      </c>
-      <c r="G80" s="41" t="inlineStr">
-        <is>
-          <t>Tên gói đúng; giá đúng theo chính sách; mặc định hiển thị giá gói 1 tháng</t>
-        </is>
-      </c>
-      <c r="H80" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I80" s="42" t="n"/>
-      <c r="J80" s="42" t="n"/>
-      <c r="K80" s="42" t="n"/>
-      <c r="L80" s="42" t="n"/>
+      <c r="B80" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 14: Luồng thanh toán</t>
+        </is>
+      </c>
+      <c r="C80" s="35" t="n"/>
+      <c r="D80" s="35" t="n"/>
+      <c r="E80" s="35" t="n"/>
+      <c r="F80" s="35" t="n"/>
+      <c r="G80" s="35" t="n"/>
+      <c r="H80" s="35" t="n"/>
+      <c r="I80" s="35" t="n"/>
+      <c r="J80" s="35" t="n"/>
+      <c r="K80" s="35" t="n"/>
+      <c r="L80" s="36" t="n"/>
     </row>
     <row r="81" ht="28.35" customHeight="1" s="32">
       <c r="A81" s="39" t="inlineStr">
@@ -3755,28 +3753,29 @@
       </c>
       <c r="C81" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D81" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra ô mã khuyến mãi, link Chọn ưu đãi và trạng thái button Áp dụng</t>
+          <t>Kiểm tra click Thanh toán khi chưa nhập đủ trường bắt buộc</t>
         </is>
       </c>
       <c r="E81" s="41" t="inlineStr">
         <is>
-          <t>- Block Thông tin thanh toán đang hiển thị</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F81" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát ô mã khi rỗng (button Áp dụng)
-2. Nhập 1 ký tự vào ô mã</t>
+          <t>1. Bỏ trống ít nhất 1 trường bắt buộc
+2. Click button Thanh toán</t>
         </is>
       </c>
       <c r="G81" s="41" t="inlineStr">
         <is>
-          <t>Ô input placeholder "Nhập mã khuyến mãi" + link "Chọn ưu đãi" (badge số) + button Áp dụng: disable khi rỗng, enable khi có ký tự</t>
+          <t>Hiển thị lỗi ở các trường bắt buộc; không thực hiện thanh toán</t>
         </is>
       </c>
       <c r="H81" s="40" t="inlineStr">
@@ -3801,27 +3800,30 @@
       </c>
       <c r="C82" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D82" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click link Chọn ưu đãi mở danh sách ưu đãi</t>
+          <t>Kiểm tra thanh toán với PTTT = COD</t>
         </is>
       </c>
       <c r="E82" s="41" t="inlineStr">
         <is>
-          <t>- Có ưu đãi đang hoạt động</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F82" s="41" t="inlineStr">
         <is>
-          <t>1. Click link "Chọn ưu đãi"</t>
+          <t>1. Nhập đầy đủ trường bắt buộc
+2. Chọn PTTT = COD
+3. Click Thanh toán</t>
         </is>
       </c>
       <c r="G82" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị danh sách ưu đãi khả dụng; badge đúng số lượng ưu đãi</t>
+          <t>Điều hướng màn hình Hoàn tất đơn hàng với trạng thái "Chưa thanh toán"</t>
         </is>
       </c>
       <c r="H82" s="40" t="inlineStr">
@@ -3851,24 +3853,25 @@
       </c>
       <c r="D83" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra áp dụng mã khuyến mãi hợp lệ</t>
+          <t>Kiểm tra thanh toán với PTTT Online điều hướng sang cổng 3rd party</t>
         </is>
       </c>
       <c r="E83" s="41" t="inlineStr">
         <is>
-          <t>- Có mã khuyến mãi hợp lệ đang hoạt động</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F83" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập mã khuyến mãi hợp lệ
-2. Click Áp dụng
-3. Quan sát Cần thanh toán</t>
+          <t>1. Nhập đầy đủ trường bắt buộc
+2. Chọn PTTT Online (VD: thẻ ATM/Visa)
+3. Click Thanh toán</t>
         </is>
       </c>
       <c r="G83" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị giá trị giảm; Cần thanh toán = giá gốc − giá trị giảm (cập nhật đúng)</t>
+          <t>Điều hướng sang màn hình thanh toán của 3rd party tương ứng, hiển thị đúng số tiền cần thanh toán</t>
         </is>
       </c>
       <c r="H83" s="40" t="inlineStr">
@@ -3898,23 +3901,25 @@
       </c>
       <c r="D84" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra áp dụng mã khuyến mãi không hợp lệ/hết hạn</t>
+          <t>Kiểm tra double-click button Thanh toán không tạo trùng đơn</t>
         </is>
       </c>
       <c r="E84" s="41" t="inlineStr">
         <is>
-          <t>- Mã khuyến mãi không tồn tại hoặc đã hết hạn</t>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
         </is>
       </c>
       <c r="F84" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập mã không hợp lệ/hết hạn
-2. Click Áp dụng</t>
+          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT Online
+2. Double-click button Thanh toán
+3. Kiểm tra log/đơn hàng tạo ra</t>
         </is>
       </c>
       <c r="G84" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị thông báo lỗi (mã không hợp lệ/hết hạn); Cần thanh toán không thay đổi</t>
+          <t>Hệ thống chỉ tạo 1 đơn hàng đúng thông tin, không bị double</t>
         </is>
       </c>
       <c r="H84" s="40" t="inlineStr">
@@ -3928,21 +3933,52 @@
       <c r="L84" s="42" t="n"/>
     </row>
     <row r="85" ht="15" customHeight="1" s="32">
-      <c r="B85" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 15: Luồng thanh toán</t>
-        </is>
-      </c>
-      <c r="C85" s="35" t="n"/>
-      <c r="D85" s="35" t="n"/>
-      <c r="E85" s="35" t="n"/>
-      <c r="F85" s="35" t="n"/>
-      <c r="G85" s="35" t="n"/>
-      <c r="H85" s="35" t="n"/>
-      <c r="I85" s="35" t="n"/>
-      <c r="J85" s="35" t="n"/>
-      <c r="K85" s="35" t="n"/>
-      <c r="L85" s="36" t="n"/>
+      <c r="A85" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B85" s="40">
+        <f>IF(D85="","",$D$3&amp;"."&amp;COUNTA($D$10:D85)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C85" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D85" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra click Thanh toán khi quá session checkout (20 phút)</t>
+        </is>
+      </c>
+      <c r="E85" s="41" t="inlineStr">
+        <is>
+          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
+- Đang ở màn hình Checkout</t>
+        </is>
+      </c>
+      <c r="F85" s="41" t="inlineStr">
+        <is>
+          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT Online
+2. Chờ hơn 20 phút
+3. Click Thanh toán</t>
+        </is>
+      </c>
+      <c r="G85" s="41" t="inlineStr">
+        <is>
+          <t>Hiển thị thông báo lỗi hợp lý; đẩy thông tin KH tiềm năng</t>
+        </is>
+      </c>
+      <c r="H85" s="40" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I85" s="42" t="n"/>
+      <c r="J85" s="42" t="n"/>
+      <c r="K85" s="42" t="n"/>
+      <c r="L85" s="42" t="n"/>
     </row>
     <row r="86" ht="41.75" customHeight="1" s="32">
       <c r="A86" s="39" t="inlineStr">
@@ -3956,34 +3992,32 @@
       </c>
       <c r="C86" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D86" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click Thanh toán khi chưa nhập đủ trường bắt buộc</t>
+          <t>Kiểm tra hết countdown thanh toán ở cổng 3rd party (~15 phút)</t>
         </is>
       </c>
       <c r="E86" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
         </is>
       </c>
       <c r="F86" s="41" t="inlineStr">
         <is>
-          <t>1. Bỏ trống ít nhất 1 trường bắt buộc
-2. Click button Thanh toán</t>
+          <t>1. Chờ hết thời gian thanh toán của kênh (~15 phút)</t>
         </is>
       </c>
       <c r="G86" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị lỗi ở các trường bắt buộc; không thực hiện thanh toán</t>
+          <t>Quay về tongdaiwifi và hiển thị màn hình không thành công</t>
         </is>
       </c>
       <c r="H86" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I86" s="42" t="n"/>
@@ -4003,35 +4037,32 @@
       </c>
       <c r="C87" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D87" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra thanh toán với PTTT = COD</t>
+          <t>Kiểm tra back từ cổng 3rd party về màn hình thanh toán</t>
         </is>
       </c>
       <c r="E87" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
         </is>
       </c>
       <c r="F87" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập đầy đủ trường bắt buộc
-2. Chọn PTTT = COD
-3. Click Thanh toán</t>
+          <t>1. Click icon back trên trình duyệt</t>
         </is>
       </c>
       <c r="G87" s="41" t="inlineStr">
         <is>
-          <t>Điều hướng màn hình Hoàn tất đơn hàng với trạng thái "Chưa thanh toán"</t>
+          <t>Về màn hình dịch vụ; disable các thông tin, chỉ cho cập nhật PTTT và mã ưu đãi</t>
         </is>
       </c>
       <c r="H87" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I87" s="42" t="n"/>
@@ -4056,30 +4087,27 @@
       </c>
       <c r="D88" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra thanh toán với PTTT Online điều hướng sang cổng 3rd party</t>
+          <t>Kiểm tra hủy/thanh toán thất bại tại cổng 3rd party</t>
         </is>
       </c>
       <c r="E88" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
         </is>
       </c>
       <c r="F88" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập đầy đủ trường bắt buộc
-2. Chọn PTTT Online (VD: thẻ ATM/Visa)
-3. Click Thanh toán</t>
+          <t>1. Hủy thanh toán hoặc nhập sai thông tin thẻ nhiều lần</t>
         </is>
       </c>
       <c r="G88" s="41" t="inlineStr">
         <is>
-          <t>Điều hướng sang màn hình thanh toán của 3rd party tương ứng, hiển thị đúng số tiền cần thanh toán</t>
+          <t>Quay về tongdaiwifi, hiển thị màn hình không thành công; đẩy KHTN</t>
         </is>
       </c>
       <c r="H88" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I88" s="42" t="n"/>
@@ -4104,25 +4132,23 @@
       </c>
       <c r="D89" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra double-click button Thanh toán không tạo trùng đơn</t>
+          <t>Kiểm tra click Thanh toán khi chính sách gói đã hết hiệu lực</t>
         </is>
       </c>
       <c r="E89" s="41" t="inlineStr">
         <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
+          <t>- Gói có ít nhất 1 chính sách đã hết hiệu lực trên QLCS</t>
         </is>
       </c>
       <c r="F89" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT Online
-2. Double-click button Thanh toán
-3. Kiểm tra log/đơn hàng tạo ra</t>
+          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT
+2. Click Thanh toán</t>
         </is>
       </c>
       <c r="G89" s="41" t="inlineStr">
         <is>
-          <t>Hệ thống chỉ tạo 1 đơn hàng đúng thông tin, không bị double</t>
+          <t>Hệ thống hiển thị thông báo lỗi, không lên đơn hàng</t>
         </is>
       </c>
       <c r="H89" s="40" t="inlineStr">
@@ -4136,52 +4162,21 @@
       <c r="L89" s="42" t="n"/>
     </row>
     <row r="90" ht="41.75" customHeight="1" s="32">
-      <c r="A90" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B90" s="40">
-        <f>IF(D90="","",$D$3&amp;"."&amp;COUNTA($D$10:D90)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C90" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D90" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra click Thanh toán khi quá session checkout (20 phút)</t>
-        </is>
-      </c>
-      <c r="E90" s="41" t="inlineStr">
-        <is>
-          <t>- Đã chọn 1 gói dịch vụ (có Địa chỉ lắp đặt) ở màn Chi tiết
-- Đang ở màn hình Checkout</t>
-        </is>
-      </c>
-      <c r="F90" s="41" t="inlineStr">
-        <is>
-          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT Online
-2. Chờ hơn 20 phút
-3. Click Thanh toán</t>
-        </is>
-      </c>
-      <c r="G90" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị thông báo lỗi hợp lý; đẩy thông tin KH tiềm năng</t>
-        </is>
-      </c>
-      <c r="H90" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I90" s="42" t="n"/>
-      <c r="J90" s="42" t="n"/>
-      <c r="K90" s="42" t="n"/>
-      <c r="L90" s="42" t="n"/>
+      <c r="B90" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 15: Màn hình Hoàn tất đơn hàng</t>
+        </is>
+      </c>
+      <c r="C90" s="35" t="n"/>
+      <c r="D90" s="35" t="n"/>
+      <c r="E90" s="35" t="n"/>
+      <c r="F90" s="35" t="n"/>
+      <c r="G90" s="35" t="n"/>
+      <c r="H90" s="35" t="n"/>
+      <c r="I90" s="35" t="n"/>
+      <c r="J90" s="35" t="n"/>
+      <c r="K90" s="35" t="n"/>
+      <c r="L90" s="36" t="n"/>
     </row>
     <row r="91" ht="28.35" customHeight="1" s="32">
       <c r="A91" s="39" t="inlineStr">
@@ -4195,32 +4190,32 @@
       </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D91" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hết countdown thanh toán ở cổng 3rd party (~15 phút)</t>
+          <t>Kiểm tra hiển thị Mã đơn hàng và hyperlink Theo dõi ĐH</t>
         </is>
       </c>
       <c r="E91" s="41" t="inlineStr">
         <is>
-          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
+          <t>- Đã hoàn tất đơn hàng thành công</t>
         </is>
       </c>
       <c r="F91" s="41" t="inlineStr">
         <is>
-          <t>1. Chờ hết thời gian thanh toán của kênh (~15 phút)</t>
+          <t>1. Quan sát khu vực Mã đơn hàng</t>
         </is>
       </c>
       <c r="G91" s="41" t="inlineStr">
         <is>
-          <t>Quay về tongdaiwifi và hiển thị màn hình không thành công</t>
+          <t>Hiển thị "Mã đơn hàng: &lt;mã&gt;" kèm hyperlink "Theo dõi ĐH"</t>
         </is>
       </c>
       <c r="H91" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I91" s="42" t="n"/>
@@ -4245,27 +4240,27 @@
       </c>
       <c r="D92" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra back từ cổng 3rd party về màn hình thanh toán</t>
+          <t>Kiểm tra click hyperlink Theo dõi đơn hàng</t>
         </is>
       </c>
       <c r="E92" s="41" t="inlineStr">
         <is>
-          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
+          <t>- Đang ở màn hình Hoàn tất đơn hàng</t>
         </is>
       </c>
       <c r="F92" s="41" t="inlineStr">
         <is>
-          <t>1. Click icon back trên trình duyệt</t>
+          <t>1. Click hyperlink Theo dõi đơn hàng</t>
         </is>
       </c>
       <c r="G92" s="41" t="inlineStr">
         <is>
-          <t>Về màn hình dịch vụ; disable các thông tin, chỉ cho cập nhật PTTT và mã ưu đãi</t>
+          <t>Điều hướng đến màn hình theo dõi đơn hàng</t>
         </is>
       </c>
       <c r="H92" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I92" s="42" t="n"/>
@@ -4285,32 +4280,33 @@
       </c>
       <c r="C93" s="40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D93" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hủy/thanh toán thất bại tại cổng 3rd party</t>
+          <t>Kiểm tra hiển thị và thu gọn/mở rộng block Thông tin khách hàng &amp; Thông tin thanh toán</t>
         </is>
       </c>
       <c r="E93" s="41" t="inlineStr">
         <is>
-          <t>- Đã điều hướng sang cổng thanh toán 3rd party</t>
+          <t>- Đang ở màn hình Hoàn tất đơn hàng</t>
         </is>
       </c>
       <c r="F93" s="41" t="inlineStr">
         <is>
-          <t>1. Hủy thanh toán hoặc nhập sai thông tin thẻ nhiều lần</t>
+          <t>1. Quan sát thông tin 2 block
+2. Thu gọn/mở rộng từng block</t>
         </is>
       </c>
       <c r="G93" s="41" t="inlineStr">
         <is>
-          <t>Quay về tongdaiwifi, hiển thị màn hình không thành công; đẩy KHTN</t>
+          <t>Hiển thị đúng thông tin đã nhập ở các bước trước; thu gọn/mở rộng hoạt động, icon đổi v ↔ ^</t>
         </is>
       </c>
       <c r="H93" s="40" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I93" s="42" t="n"/>
@@ -4335,23 +4331,22 @@
       </c>
       <c r="D94" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click Thanh toán khi chính sách gói đã hết hiệu lực</t>
+          <t>Kiểm tra trạng thái hoàn tất với COD và Online</t>
         </is>
       </c>
       <c r="E94" s="41" t="inlineStr">
         <is>
-          <t>- Gói có ít nhất 1 chính sách đã hết hiệu lực trên QLCS</t>
+          <t>- Hoàn tất qua COD hoặc Online thành công</t>
         </is>
       </c>
       <c r="F94" s="41" t="inlineStr">
         <is>
-          <t>1. Nhập đầy đủ trường bắt buộc, chọn PTTT
-2. Click Thanh toán</t>
+          <t>1. Quan sát label trạng thái trên màn Hoàn tất</t>
         </is>
       </c>
       <c r="G94" s="41" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi, không lên đơn hàng</t>
+          <t>COD → "Chưa thanh toán"; Online thành công → "Thanh toán thành công"; các bước header màu xanh lá</t>
         </is>
       </c>
       <c r="H94" s="40" t="inlineStr">
@@ -4365,66 +4360,67 @@
       <c r="L94" s="42" t="n"/>
     </row>
     <row r="95" ht="15" customHeight="1" s="32">
-      <c r="B95" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 16: Màn hình Hoàn tất đơn hàng</t>
-        </is>
-      </c>
-      <c r="C95" s="35" t="n"/>
-      <c r="D95" s="35" t="n"/>
-      <c r="E95" s="35" t="n"/>
-      <c r="F95" s="35" t="n"/>
-      <c r="G95" s="35" t="n"/>
-      <c r="H95" s="35" t="n"/>
-      <c r="I95" s="35" t="n"/>
-      <c r="J95" s="35" t="n"/>
-      <c r="K95" s="35" t="n"/>
-      <c r="L95" s="36" t="n"/>
+      <c r="A95" s="39" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="B95" s="40">
+        <f>IF(D95="","",$D$3&amp;"."&amp;COUNTA($D$10:D95)&amp;"")</f>
+        <v/>
+      </c>
+      <c r="C95" s="40" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D95" s="41" t="inlineStr">
+        <is>
+          <t>Kiểm tra đối soát đơn hàng và hợp đồng sau thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="E95" s="41" t="inlineStr">
+        <is>
+          <t>- Đã thanh toán thành công</t>
+        </is>
+      </c>
+      <c r="F95" s="41" t="inlineStr">
+        <is>
+          <t>1. Truy cập web-admin kiểm tra đơn hàng
+2. Truy cập inside kiểm tra hợp đồng</t>
+        </is>
+      </c>
+      <c r="G95" s="41" t="inlineStr">
+        <is>
+          <t>Đơn hàng ghi nhận đúng thông tin đã nhập; Hợp đồng ghi nhận đúng thông tin đơn hàng</t>
+        </is>
+      </c>
+      <c r="H95" s="40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="I95" s="42" t="n"/>
+      <c r="J95" s="42" t="n"/>
+      <c r="K95" s="42" t="n"/>
+      <c r="L95" s="42" t="n"/>
     </row>
     <row r="96" ht="28.35" customHeight="1" s="32">
-      <c r="A96" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B96" s="40">
-        <f>IF(D96="","",$D$3&amp;"."&amp;COUNTA($D$10:D96)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C96" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D96" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra hiển thị Mã đơn hàng và hyperlink Theo dõi ĐH</t>
-        </is>
-      </c>
-      <c r="E96" s="41" t="inlineStr">
-        <is>
-          <t>- Đã hoàn tất đơn hàng thành công</t>
-        </is>
-      </c>
-      <c r="F96" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát khu vực Mã đơn hàng</t>
-        </is>
-      </c>
-      <c r="G96" s="41" t="inlineStr">
-        <is>
-          <t>Hiển thị "Mã đơn hàng: &lt;mã&gt;" kèm hyperlink "Theo dõi ĐH"</t>
-        </is>
-      </c>
-      <c r="H96" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I96" s="42" t="n"/>
-      <c r="J96" s="42" t="n"/>
-      <c r="K96" s="42" t="n"/>
-      <c r="L96" s="42" t="n"/>
+      <c r="B96" s="38" t="inlineStr">
+        <is>
+          <t>Nhóm 16: Empty/Error state, Quyền truy cập &amp; Mobile (Mandatory)</t>
+        </is>
+      </c>
+      <c r="C96" s="35" t="n"/>
+      <c r="D96" s="35" t="n"/>
+      <c r="E96" s="35" t="n"/>
+      <c r="F96" s="35" t="n"/>
+      <c r="G96" s="35" t="n"/>
+      <c r="H96" s="35" t="n"/>
+      <c r="I96" s="35" t="n"/>
+      <c r="J96" s="35" t="n"/>
+      <c r="K96" s="35" t="n"/>
+      <c r="L96" s="36" t="n"/>
     </row>
     <row r="97" ht="28.35" customHeight="1" s="32">
       <c r="A97" s="39" t="inlineStr">
@@ -4443,22 +4439,23 @@
       </c>
       <c r="D97" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra click hyperlink Theo dõi đơn hàng</t>
+          <t>Kiểm tra truy cập màn hình Checkout khi chưa đăng nhập (guest)</t>
         </is>
       </c>
       <c r="E97" s="41" t="inlineStr">
         <is>
-          <t>- Đang ở màn hình Hoàn tất đơn hàng</t>
+          <t>- Chưa đăng nhập tài khoản; có link đăng ký dịch vụ</t>
         </is>
       </c>
       <c r="F97" s="41" t="inlineStr">
         <is>
-          <t>1. Click hyperlink Theo dõi đơn hàng</t>
+          <t>1. Mở link đăng ký dịch vụ ở trạng thái chưa đăng nhập
+2. Thực hiện checkout</t>
         </is>
       </c>
       <c r="G97" s="41" t="inlineStr">
         <is>
-          <t>Điều hướng đến màn hình theo dõi đơn hàng</t>
+          <t>Cho phép checkout ở trạng thái guest (luồng đăng ký dịch vụ không bắt buộc đăng nhập)</t>
         </is>
       </c>
       <c r="H97" s="40" t="inlineStr">
@@ -4488,28 +4485,27 @@
       </c>
       <c r="D98" s="41" t="inlineStr">
         <is>
-          <t>Kiểm tra hiển thị và thu gọn/mở rộng block Thông tin khách hàng &amp; Thông tin thanh toán</t>
+          <t>Kiểm tra hiển thị màn hình Checkout trên mobile (≤ 768px)</t>
         </is>
       </c>
       <c r="E98" s="41" t="inlineStr">
         <is>
-          <t>- Đang ở màn hình Hoàn tất đơn hàng</t>
+          <t>- Mở màn hình Checkout trên viewport ≤ 768px</t>
         </is>
       </c>
       <c r="F98" s="41" t="inlineStr">
         <is>
-          <t>1. Quan sát thông tin 2 block
-2. Thu gọn/mở rộng từng block</t>
+          <t>1. Quan sát layout tổng thể các block trên mobile</t>
         </is>
       </c>
       <c r="G98" s="41" t="inlineStr">
         <is>
-          <t>Hiển thị đúng thông tin đã nhập ở các bước trước; thu gọn/mở rộng hoạt động, icon đổi v ↔ ^</t>
+          <t>Các block hiển thị đúng, không vỡ layout, không tràn ngang; các trường/button thao tác được</t>
         </is>
       </c>
       <c r="H98" s="40" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I98" s="42" t="n"/>
@@ -4517,329 +4513,40 @@
       <c r="K98" s="42" t="n"/>
       <c r="L98" s="42" t="n"/>
     </row>
-    <row r="99" ht="28.35" customHeight="1" s="32">
-      <c r="A99" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B99" s="40">
-        <f>IF(D99="","",$D$3&amp;"."&amp;COUNTA($D$10:D99)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C99" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D99" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra trạng thái hoàn tất với COD và Online</t>
-        </is>
-      </c>
-      <c r="E99" s="41" t="inlineStr">
-        <is>
-          <t>- Hoàn tất qua COD hoặc Online thành công</t>
-        </is>
-      </c>
-      <c r="F99" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát label trạng thái trên màn Hoàn tất</t>
-        </is>
-      </c>
-      <c r="G99" s="41" t="inlineStr">
-        <is>
-          <t>COD → "Chưa thanh toán"; Online thành công → "Thanh toán thành công"; các bước header màu xanh lá</t>
-        </is>
-      </c>
-      <c r="H99" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I99" s="42" t="n"/>
-      <c r="J99" s="42" t="n"/>
-      <c r="K99" s="42" t="n"/>
-      <c r="L99" s="42" t="n"/>
-    </row>
-    <row r="100" ht="28.35" customHeight="1" s="32">
-      <c r="A100" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B100" s="40">
-        <f>IF(D100="","",$D$3&amp;"."&amp;COUNTA($D$10:D100)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C100" s="40" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D100" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra đối soát đơn hàng và hợp đồng sau thanh toán thành công</t>
-        </is>
-      </c>
-      <c r="E100" s="41" t="inlineStr">
-        <is>
-          <t>- Đã thanh toán thành công</t>
-        </is>
-      </c>
-      <c r="F100" s="41" t="inlineStr">
-        <is>
-          <t>1. Truy cập web-admin kiểm tra đơn hàng
-2. Truy cập inside kiểm tra hợp đồng</t>
-        </is>
-      </c>
-      <c r="G100" s="41" t="inlineStr">
-        <is>
-          <t>Đơn hàng ghi nhận đúng thông tin đã nhập; Hợp đồng ghi nhận đúng thông tin đơn hàng</t>
-        </is>
-      </c>
-      <c r="H100" s="40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I100" s="42" t="n"/>
-      <c r="J100" s="42" t="n"/>
-      <c r="K100" s="42" t="n"/>
-      <c r="L100" s="42" t="n"/>
-    </row>
-    <row r="101" ht="15" customHeight="1" s="32">
-      <c r="B101" s="38" t="inlineStr">
-        <is>
-          <t>Nhóm 17: Empty/Error state, Quyền truy cập &amp; Mobile (Mandatory)</t>
-        </is>
-      </c>
-      <c r="C101" s="35" t="n"/>
-      <c r="D101" s="35" t="n"/>
-      <c r="E101" s="35" t="n"/>
-      <c r="F101" s="35" t="n"/>
-      <c r="G101" s="35" t="n"/>
-      <c r="H101" s="35" t="n"/>
-      <c r="I101" s="35" t="n"/>
-      <c r="J101" s="35" t="n"/>
-      <c r="K101" s="35" t="n"/>
-      <c r="L101" s="36" t="n"/>
-    </row>
-    <row r="102" ht="28.35" customHeight="1" s="32">
-      <c r="A102" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B102" s="40">
-        <f>IF(D102="","",$D$3&amp;"."&amp;COUNTA($D$10:D102)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C102" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D102" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra truy cập màn hình Checkout khi chưa đăng nhập (guest)</t>
-        </is>
-      </c>
-      <c r="E102" s="41" t="inlineStr">
-        <is>
-          <t>- Chưa đăng nhập tài khoản; có link đăng ký dịch vụ</t>
-        </is>
-      </c>
-      <c r="F102" s="41" t="inlineStr">
-        <is>
-          <t>1. Mở link đăng ký dịch vụ ở trạng thái chưa đăng nhập
-2. Thực hiện checkout</t>
-        </is>
-      </c>
-      <c r="G102" s="41" t="inlineStr">
-        <is>
-          <t>Cho phép checkout ở trạng thái guest (luồng đăng ký dịch vụ không bắt buộc đăng nhập)</t>
-        </is>
-      </c>
-      <c r="H102" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I102" s="42" t="n"/>
-      <c r="J102" s="42" t="n"/>
-      <c r="K102" s="42" t="n"/>
-      <c r="L102" s="42" t="n"/>
-    </row>
-    <row r="103" ht="41.75" customHeight="1" s="32">
-      <c r="A103" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B103" s="40">
-        <f>IF(D103="","",$D$3&amp;"."&amp;COUNTA($D$10:D103)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C103" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D103" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra Block Phương thức thanh toán khi chính sách không khai báo PTTT nào</t>
-        </is>
-      </c>
-      <c r="E103" s="41" t="inlineStr">
-        <is>
-          <t>- Gói có chính sách nhưng không khai báo PTTT nào</t>
-        </is>
-      </c>
-      <c r="F103" s="41" t="inlineStr">
-        <is>
-          <t>1. Truy cập Checkout của gói này
-2. Quan sát Block Phương thức thanh toán</t>
-        </is>
-      </c>
-      <c r="G103" s="41" t="inlineStr">
-        <is>
-          <t>[BLOCKED – cần confirm: khi chính sách không khai báo PTTT nào thì Block Phương thức thanh toán hiển thị thế nào (ẩn/placeholder/thông báo) và có cho thanh toán không?]</t>
-        </is>
-      </c>
-      <c r="H103" s="40" t="n"/>
-      <c r="I103" s="42" t="n"/>
-      <c r="J103" s="42" t="n"/>
-      <c r="K103" s="42" t="n"/>
-      <c r="L103" s="42" t="inlineStr">
-        <is>
-          <t>Bỏ case này giúp tôi, case này không xảy ra</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="28.35" customHeight="1" s="32">
-      <c r="A104" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B104" s="40">
-        <f>IF(D104="","",$D$3&amp;"."&amp;COUNTA($D$10:D104)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C104" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D104" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra xử lý khi API chính sách lỗi/timeout lúc kiểm tra giá</t>
-        </is>
-      </c>
-      <c r="E104" s="41" t="inlineStr">
-        <is>
-          <t>- Block Địa chỉ lắp đặt đang hiển thị</t>
-        </is>
-      </c>
-      <c r="F104" s="41" t="inlineStr">
-        <is>
-          <t>1. Chọn đủ địa chỉ để trigger API chính sách
-2. Giả lập API chính sách lỗi/timeout</t>
-        </is>
-      </c>
-      <c r="G104" s="41" t="inlineStr">
-        <is>
-          <t>[BLOCKED – cần confirm: hành vi khi API chính sách lỗi/timeout — hiển thị thông báo gì, có chặn bước thanh toán không?]</t>
-        </is>
-      </c>
-      <c r="H104" s="40" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I104" s="42" t="n"/>
-      <c r="J104" s="42" t="n"/>
-      <c r="K104" s="42" t="n"/>
-      <c r="L104" s="42" t="inlineStr">
-        <is>
-          <t>Bỏ case này giúp tôi, case này không xảy ra</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="28.35" customHeight="1" s="32">
-      <c r="A105" s="39" t="inlineStr">
-        <is>
-          <t>AI</t>
-        </is>
-      </c>
-      <c r="B105" s="40">
-        <f>IF(D105="","",$D$3&amp;"."&amp;COUNTA($D$10:D105)&amp;"")</f>
-        <v/>
-      </c>
-      <c r="C105" s="40" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D105" s="41" t="inlineStr">
-        <is>
-          <t>Kiểm tra hiển thị màn hình Checkout trên mobile (≤ 768px)</t>
-        </is>
-      </c>
-      <c r="E105" s="41" t="inlineStr">
-        <is>
-          <t>- Mở màn hình Checkout trên viewport ≤ 768px</t>
-        </is>
-      </c>
-      <c r="F105" s="41" t="inlineStr">
-        <is>
-          <t>1. Quan sát layout tổng thể các block trên mobile</t>
-        </is>
-      </c>
-      <c r="G105" s="41" t="inlineStr">
-        <is>
-          <t>Các block hiển thị đúng, không vỡ layout, không tràn ngang; các trường/button thao tác được</t>
-        </is>
-      </c>
-      <c r="H105" s="40" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="I105" s="42" t="n"/>
-      <c r="J105" s="42" t="n"/>
-      <c r="K105" s="42" t="n"/>
-      <c r="L105" s="42" t="n"/>
-    </row>
+    <row r="99" ht="28.35" customHeight="1" s="32"/>
+    <row r="100" ht="28.35" customHeight="1" s="32"/>
+    <row r="101" ht="15" customHeight="1" s="32"/>
+    <row r="102" ht="28.35" customHeight="1" s="32"/>
+    <row r="103" ht="41.75" customHeight="1" s="32"/>
+    <row r="104" ht="28.35" customHeight="1" s="32"/>
+    <row r="105" ht="28.35" customHeight="1" s="32"/>
   </sheetData>
-  <mergeCells count="26">
-    <mergeCell ref="B50:L50"/>
-    <mergeCell ref="B16:L16"/>
-    <mergeCell ref="B72:L72"/>
-    <mergeCell ref="B59:L59"/>
+  <mergeCells count="25">
+    <mergeCell ref="B90:L90"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="G7:G8"/>
-    <mergeCell ref="B31:L31"/>
-    <mergeCell ref="B18:L18"/>
+    <mergeCell ref="B46:L46"/>
+    <mergeCell ref="B27:L27"/>
+    <mergeCell ref="B96:L96"/>
     <mergeCell ref="D7:D8"/>
     <mergeCell ref="H7:H8"/>
-    <mergeCell ref="B101:L101"/>
-    <mergeCell ref="B57:L57"/>
+    <mergeCell ref="B14:L14"/>
     <mergeCell ref="B53:L53"/>
-    <mergeCell ref="B44:L44"/>
-    <mergeCell ref="B78:L78"/>
+    <mergeCell ref="B73:L73"/>
     <mergeCell ref="C7:C8"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="I7:L7"/>
+    <mergeCell ref="B40:L40"/>
     <mergeCell ref="B9:L9"/>
+    <mergeCell ref="B49:L49"/>
     <mergeCell ref="B68:L68"/>
-    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="B64:L64"/>
+    <mergeCell ref="B55:L55"/>
+    <mergeCell ref="B80:L80"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B95:L95"/>
+    <mergeCell ref="B20:L20"/>
     <mergeCell ref="F7:F8"/>
-    <mergeCell ref="B36:L36"/>
-    <mergeCell ref="B85:L85"/>
+    <mergeCell ref="B32:L32"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -7628,7 +7335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L31"/>
+  <dimension ref="A3:L31"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="31" min="1" max="1"/>
@@ -7644,8 +7351,6 @@
     <col width="22.3" customWidth="1" style="31" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="32">
       <c r="C3" s="44" t="inlineStr">
         <is>
@@ -7670,8 +7375,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7" ht="30" customHeight="1" s="32">
       <c r="A7" s="45" t="inlineStr">
         <is>

</xml_diff>